<commit_message>
v2 budget: note what the TMP117 can and cannot resolve
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1g5ouZCd4fvcL4KzTMSdf
</commit_message>
<xml_diff>
--- a/docs/v2-budget/STM_v2_budget.xlsx
+++ b/docs/v2-budget/STM_v2_budget.xlsx
@@ -526,7 +526,7 @@
     <t xml:space="preserve">https://adafruit.com/product/4821</t>
   </si>
   <si>
-    <t xml:space="preserve">Direct product page. Zahl: monitor temperature; Baird: steady amplifier temperature.</t>
+    <t xml:space="preserve">Direct product page, in stock. Checked 2026-10-21: resolution 0.0078 C per step, accuracy +/-0.1 C. Resolution is what matters, since this is for spotting changes, not absolute temperature. A printed loop expands roughly 1 nm per mK (assumes 30-70 ppm/K, about 30 mm of mismatched plastic, not measured), so one step is about 10 nm of drift. Good enough to tell whether drift of tens of nm follows temperature and when the head has settled; no affordable sensor resolves the ~0.1 mK that atom-scale drift corresponds to. Keep its I2C wiring away from the preamp input, or log it standalone (INVENTORY.md). Zahl: monitor temperature; Baird: steady amplifier temperature.</t>
   </si>
   <si>
     <t xml:space="preserve">ME-01</t>
@@ -4109,7 +4109,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
         <v>161</v>
       </c>

</xml_diff>

<commit_message>
v2 budget: FAS200 2 in screws at catalog price, add F25SSN1 bushings
Total now $1,817.94.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1g5ouZCd4fvcL4KzTMSdf
</commit_message>
<xml_diff>
--- a/docs/v2-budget/STM_v2_budget.xlsx
+++ b/docs/v2-budget/STM_v2_budget.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="839" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="597">
   <si>
     <t xml:space="preserve">STM v2 (UCSD) - budget summary, lean scenario</t>
   </si>
@@ -268,7 +268,7 @@
     <t xml:space="preserve">PZ-04</t>
   </si>
   <si>
-    <t xml:space="preserve">Fine-pitch adjuster screws, 1/4-80 (one motor-driven, two hand-set)</t>
+    <t xml:space="preserve">Ultra-fine adjustment screws, 1/4-80, 2 in long (one motor-driven, two hand-set)</t>
   </si>
   <si>
     <t xml:space="preserve">Thorlabs FAS200</t>
@@ -280,30 +280,45 @@
     <t xml:space="preserve">https://www.thorlabs.com/thorproduct.cfm?partnumber=FAS200</t>
   </si>
   <si>
+    <t xml:space="preserve">Jacob specified FAS200 (2 in, 1/4-80), the same screws v1 used (three bought 2026-06-24 at $8.78). $8.80 is the Thorlabs catalog page 521 price (PDF loaded; undated); the product page does not load from here. 1/4-80 is 317.5 um per turn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PZ-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Threaded bushings for the 1/4-80 screws (one per screw)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thorlabs F25SSN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.thorlabs.com/thorproduct.cfm?partnumber=F25SSN1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/4-80 threaded bushing, 0.63 in long, from the same Thorlabs catalog page ($8.60). Gives each screw a metal thread instead of a printed one, which wears. The printed part needs a hole sized to the bushing (take it from the Thorlabs drawing). v1's CAD names McMaster 98625A960 brass inserts instead; McMaster does not load here, so not priced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controller board, fully assembled (v1 design)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JLCPCB SMT assembly, v1 controller design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JLCPCB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://jlcpcb.com/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">each (2 min)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Historical - v1 receipt</t>
   </si>
   <si>
-    <t xml:space="preserve">Same screws as v1 (three bought 2026-06-24 at $8.78). Thorlabs pages do not load from here, so this is v1's price. 1/4-80 is 317.5 um per turn. v1 ran them in printed threads; matching brass bushings are not priced (U6).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EL-01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controller board, fully assembled (v1 design)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JLCPCB SMT assembly, v1 controller design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JLCPCB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://jlcpcb.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">each (2 min)</t>
-  </si>
-  <si>
     <t xml:space="preserve">v1 invoice 2026-07-15 unit price. Re-quote not possible from here: JLCPCB prices only after gerber + BOM upload. Parts prices have moved since (e.g. LT1469 now $23.77 and out of stock at LCSC).</t>
   </si>
   <si>
@@ -970,7 +985,7 @@
     <t xml:space="preserve">Jacob's choice (2026-10-21): a stepper-driven fine screw, not stick-slip. v1's rubber-band/spring plate and geared 28BYJ-48 are retired.</t>
   </si>
   <si>
-    <t xml:space="preserve">Chosen: stepper on a 1/4-80 screw = PZ-02 + PZ-03 + PZ-04</t>
+    <t xml:space="preserve">Chosen: stepper on a 1/4-80 screw = PZ-02 to PZ-05</t>
   </si>
   <si>
     <t xml:space="preserve">   Motor: NEMA-17 (Adafruit 324) with a TMC2209 driver at up to 1/256 microstepping, about 6 nm of screw travel per microstep before any lever</t>
@@ -1531,19 +1546,19 @@
     <t xml:space="preserve">U6</t>
   </si>
   <si>
-    <t xml:space="preserve">Screw bushings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">v1 ran the 1/4-80 screws in printed threads, which wear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None priced</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brass 1/4-80 bushings would add a few dollars each</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Price Thorlabs or Newport bushings when their pages load</t>
+    <t xml:space="preserve">Bushing fit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F25SSN1 bushings are priced, but the printed hole for them is not drawn yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bushings $25.80, priced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If the McMaster 98625A960 press-in inserts from v1's CAD are used instead, a few dollars different</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size the printed hole from the Thorlabs drawing, or price the McMaster insert</t>
   </si>
   <si>
     <t xml:space="preserve">U7</t>
@@ -1610,6 +1625,9 @@
   </si>
   <si>
     <t xml:space="preserve">PZ-04 Thorlabs FAS200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PZ-05 Thorlabs F25SSN1</t>
   </si>
   <si>
     <t xml:space="preserve">EL-01 JLCPCB SMT assembly, v1 controller design</t>
@@ -2322,7 +2340,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$34,A5,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$35,A5,'Detailed BOM'!$K$5:$K$35)</f>
         <v>131</v>
       </c>
     </row>
@@ -2331,8 +2349,8 @@
         <v>7</v>
       </c>
       <c r="B6" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$34,A6,'Detailed BOM'!$K$5:$K$34)</f>
-        <v>49.29</v>
+        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$35,A6,'Detailed BOM'!$K$5:$K$35)</f>
+        <v>75.15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2340,7 +2358,7 @@
         <v>8</v>
       </c>
       <c r="B7" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$34,A7,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$35,A7,'Detailed BOM'!$K$5:$K$35)</f>
         <v>497.06</v>
       </c>
     </row>
@@ -2349,7 +2367,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$34,A8,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$35,A8,'Detailed BOM'!$K$5:$K$35)</f>
         <v>132.5082</v>
       </c>
     </row>
@@ -2358,7 +2376,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$34,A9,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$35,A9,'Detailed BOM'!$K$5:$K$35)</f>
         <v>94.68</v>
       </c>
     </row>
@@ -2367,7 +2385,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$34,A10,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$35,A10,'Detailed BOM'!$K$5:$K$35)</f>
         <v>54.5</v>
       </c>
     </row>
@@ -2376,7 +2394,7 @@
         <v>12</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$34,A11,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$B$5:$B$35,A11,'Detailed BOM'!$K$5:$K$35)</f>
         <v>94.98</v>
       </c>
     </row>
@@ -2386,7 +2404,7 @@
       </c>
       <c r="B12" s="5" t="n">
         <f aca="false">SUM(B5:B11)</f>
-        <v>1054.0182</v>
+        <v>1079.8782</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>14</v>
@@ -2397,8 +2415,8 @@
         <v>15</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$L$5:$L$34,"Verified*",'Detailed BOM'!$K$5:$K$34)</f>
-        <v>347.0682</v>
+        <f aca="false">SUMIF('Detailed BOM'!$L$5:$L$35,"Verified*",'Detailed BOM'!$K$5:$K$35)</f>
+        <v>399.2682</v>
       </c>
       <c r="C13" s="7"/>
     </row>
@@ -2407,8 +2425,8 @@
         <v>16</v>
       </c>
       <c r="B14" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$L$5:$L$34,"Historical*",'Detailed BOM'!$K$5:$K$34)</f>
-        <v>517.58</v>
+        <f aca="false">SUMIF('Detailed BOM'!$L$5:$L$35,"Historical*",'Detailed BOM'!$K$5:$K$35)</f>
+        <v>491.24</v>
       </c>
       <c r="C14" s="7"/>
     </row>
@@ -2417,7 +2435,7 @@
         <v>17</v>
       </c>
       <c r="B15" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$L$5:$L$34,"Estimated",'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$L$5:$L$35,"Estimated",'Detailed BOM'!$K$5:$K$35)</f>
         <v>189.37</v>
       </c>
       <c r="C15" s="7"/>
@@ -2460,7 +2478,7 @@
       </c>
       <c r="B19" s="3" t="n">
         <f aca="false">'Vendor-order totals'!I20</f>
-        <v>81.6864105</v>
+        <v>83.6905605</v>
       </c>
       <c r="C19" s="7"/>
     </row>
@@ -2470,7 +2488,7 @@
       </c>
       <c r="B20" s="5" t="n">
         <f aca="false">B12+B16+B17+B18+B19</f>
-        <v>1624.8086805</v>
+        <v>1652.6728305</v>
       </c>
       <c r="C20" s="6"/>
     </row>
@@ -2480,7 +2498,7 @@
       </c>
       <c r="B21" s="3" t="n">
         <f aca="false">B20*Assumptions!B6</f>
-        <v>162.48086805</v>
+        <v>165.26728305</v>
       </c>
       <c r="C21" s="7"/>
     </row>
@@ -2490,7 +2508,7 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">B20+B21</f>
-        <v>1787.28954855</v>
+        <v>1817.94011355</v>
       </c>
       <c r="C22" s="10"/>
     </row>
@@ -2510,7 +2528,7 @@
       </c>
       <c r="B24" s="12" t="n">
         <f aca="false">Assumptions!B9-B22</f>
-        <v>212.71045145</v>
+        <v>182.05988645</v>
       </c>
       <c r="C24" s="7"/>
     </row>
@@ -2542,7 +2560,7 @@
       </c>
       <c r="B28" s="3" t="n">
         <f aca="false">'Approach options'!F14</f>
-        <v>115.0047</v>
+        <v>89.1447</v>
       </c>
       <c r="C28" s="7"/>
     </row>
@@ -2674,7 +2692,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
@@ -2683,7 +2701,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>517</v>
+        <v>522</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2696,31 +2714,31 @@
         <v>65</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>518</v>
+        <v>523</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>519</v>
+        <v>524</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>520</v>
+        <v>525</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>521</v>
+        <v>526</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2730,15 +2748,15 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="B9" s="18" t="s">
         <v>63</v>
@@ -2746,7 +2764,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="B10" s="18" t="s">
         <v>71</v>
@@ -2754,7 +2772,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="B11" s="18" t="s">
         <v>76</v>
@@ -2762,7 +2780,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="B12" s="18" t="s">
         <v>82</v>
@@ -2770,55 +2788,55 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>528</v>
+        <v>533</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>529</v>
+        <v>534</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>530</v>
+        <v>535</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>531</v>
+        <v>536</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>532</v>
+        <v>537</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>533</v>
+        <v>538</v>
       </c>
       <c r="B19" s="18" t="s">
         <v>117</v>
@@ -2826,63 +2844,63 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>534</v>
+        <v>539</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>535</v>
+        <v>540</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>536</v>
-      </c>
-      <c r="B22" s="0" t="s">
-        <v>537</v>
+        <v>541</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>538</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>141</v>
+        <v>542</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>543</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>542</v>
+        <v>547</v>
       </c>
       <c r="B27" s="18" t="s">
         <v>164</v>
@@ -2890,234 +2908,242 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>544</v>
+        <v>549</v>
       </c>
       <c r="B29" s="18" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="B30" s="18" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="B31" s="18" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="B32" s="18" t="s">
-        <v>548</v>
+        <v>196</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B33" s="18" t="s">
-        <v>452</v>
+        <v>554</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
       <c r="B34" s="18" t="s">
-        <v>551</v>
+        <v>457</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="B35" s="18" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="B36" s="18" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="B37" s="18" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="B39" s="18" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="B40" s="18" t="s">
-        <v>447</v>
+        <v>567</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>563</v>
+        <v>568</v>
       </c>
       <c r="B41" s="18" t="s">
-        <v>564</v>
+        <v>452</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="B42" s="18" t="s">
-        <v>249</v>
+        <v>570</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="B43" s="18" t="s">
-        <v>455</v>
+        <v>254</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="B44" s="18" t="s">
-        <v>241</v>
+        <v>460</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>568</v>
+        <v>573</v>
       </c>
       <c r="B45" s="18" t="s">
-        <v>569</v>
+        <v>246</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="B46" s="18" t="s">
-        <v>231</v>
+        <v>575</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>571</v>
+        <v>576</v>
       </c>
       <c r="B47" s="18" t="s">
-        <v>572</v>
+        <v>236</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B48" s="18" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B49" s="18" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="B50" s="18" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B51" s="18" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="B52" s="18" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B53" s="18" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="B54" s="18" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="B55" s="18" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>589</v>
-      </c>
-      <c r="B56" s="0" t="s">
-        <v>590</v>
+        <v>593</v>
+      </c>
+      <c r="B56" s="18" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="0" t="s">
+        <v>595</v>
+      </c>
+      <c r="B57" s="0" t="s">
+        <v>596</v>
       </c>
     </row>
   </sheetData>
@@ -3126,47 +3152,48 @@
     <hyperlink ref="B10" r:id="rId2" display="https://www.adafruit.com/product/324"/>
     <hyperlink ref="B11" r:id="rId3" display="https://adafruit.com/product/6121"/>
     <hyperlink ref="B12" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=FAS200"/>
-    <hyperlink ref="B13" r:id="rId5" display="https://jlcpcb.com/"/>
+    <hyperlink ref="B13" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=F25SSN1"/>
     <hyperlink ref="B14" r:id="rId6" display="https://jlcpcb.com/"/>
     <hyperlink ref="B15" r:id="rId7" display="https://jlcpcb.com/"/>
     <hyperlink ref="B16" r:id="rId8" display="https://jlcpcb.com/"/>
     <hyperlink ref="B17" r:id="rId9" display="https://jlcpcb.com/"/>
-    <hyperlink ref="B18" r:id="rId10" display="https://www.digikey.com/en/products/detail/analog-devices-inc/LT1469IN8-PBF/962892"/>
-    <hyperlink ref="B19" r:id="rId11" display="https://www.digikey.com/en/products/detail/ohmite/SM104031007FE/824190"/>
-    <hyperlink ref="B20" r:id="rId12" display="https://octopart.com/part/keystone/11301"/>
-    <hyperlink ref="B21" r:id="rId13" display="https://www.lcsc.com/product-detail/C50636.html"/>
-    <hyperlink ref="B23" r:id="rId14" display="https://www.jameco.com/z/182M18-Hammond-Manufacturing-Toroidal-Transformer-120VA-50Hz-Dual-Secondary-36VCT-3-33A-Series-18V-6-66A-Parallel_2575671.html"/>
-    <hyperlink ref="B24" r:id="rId15" display="https://batteryjunction.com/batteries/shop-by-size/9v/energizer-522bp-4"/>
-    <hyperlink ref="B25" r:id="rId16" display="https://octopart.com/part/keystone/1294"/>
-    <hyperlink ref="B26" r:id="rId17" display="https://www.sparkfun.com/teensy-4-1.html"/>
-    <hyperlink ref="B27" r:id="rId18" display="https://adafruit.com/product/4821"/>
-    <hyperlink ref="B28" r:id="rId19" display="https://store.sunlu.com/products/petg-cfpetg-carbon-fiber-3d-printer-filament-1kg"/>
-    <hyperlink ref="B29" r:id="rId20" display="https://www.walmart.com/ip/533082272"/>
-    <hyperlink ref="B30" r:id="rId21" display="https://www.tedpella.com/AFM_html/AFM.aspx"/>
-    <hyperlink ref="B31" r:id="rId22" display="https://www.isolateit.com/products/sorbothane-acoustic-and-vibration-isolation-square-6-x-6-pads"/>
-    <hyperlink ref="B32" r:id="rId23" display="https://jlc3dp.com/help/article/us-tariff-policy-faq"/>
-    <hyperlink ref="B33" r:id="rId24" display="https://www.piezodrive.com/?p=991"/>
-    <hyperlink ref="B34" r:id="rId25" display="https://www.piezodrive.com/piezoelectric-tube-scanners/"/>
-    <hyperlink ref="B35" r:id="rId26" display="https://www.piezodrive.com/product-category/tube-scanners/"/>
-    <hyperlink ref="B36" r:id="rId27" display="https://www.piezodrive.com/product/pdu150-three-channel-ultra-low-noise-150v-piezo-driver/"/>
-    <hyperlink ref="B37" r:id="rId28" display="https://www.piezodrive.com/product/ps1-24v-power-supply-for-modules/"/>
-    <hyperlink ref="B38" r:id="rId29" display="https://www.piezodrive.com/product/td250-six-channel-250v/"/>
-    <hyperlink ref="B39" r:id="rId30" display="https://www.piezodrive.com/product/horizontal-tube-wiring/"/>
-    <hyperlink ref="B40" r:id="rId31" display="https://trykintsugi.com/sales-tax-guides/usa/california/san-diego-county.md"/>
-    <hyperlink ref="B41" r:id="rId32" display="https://www.eevblog.com/forum/manufacture/lcscglobal-direct-shipping-to-usa-tariff-question/"/>
-    <hyperlink ref="B42" r:id="rId33" display="https://mae156b.eng.ucsd.edu/mae156-resources/mae-undergrad-lab-resources/lab-shops/ucsd-lab-shop-resources-outside-of-mae"/>
-    <hyperlink ref="B43" r:id="rId34" display="https://mpl.ucsd.edu/machine-shop-info/"/>
-    <hyperlink ref="B44" r:id="rId35" display="https://jacobsschool.ucsd.edu/envision"/>
-    <hyperlink ref="B45" r:id="rId36" display="https://www.goodfellow.com/usa/macor-glass-ceramic-rod-1000004916"/>
-    <hyperlink ref="B46" r:id="rId37" display="https://store.bruker.com/products/dpt10"/>
-    <hyperlink ref="B47" r:id="rId38" display="https://www.2spi.com/item/z01707/"/>
-    <hyperlink ref="B48" r:id="rId39" display="https://www.sigmaaldrich.com/US/en/product/aldrich/gf84004523"/>
-    <hyperlink ref="B49" r:id="rId40" display="https://www.penntoolco.com/grizzly-12-x-18-x-3-granite-surface-plate-no-ledge-g9651"/>
-    <hyperlink ref="B50" r:id="rId41" display="https://www.batterymart.com/p-energizer-la522-9volt-lithium-battery.html"/>
-    <hyperlink ref="B51" r:id="rId42" display="https://vetco.net/products/8331d-14g_silver_conductive_epoxy_adhesive_-_mg_chemicals_8331d-14g"/>
-    <hyperlink ref="B52" r:id="rId43" display="https://kozakmicro.com/collections/1-4-80-tpi-oem-alternative-screws"/>
-    <hyperlink ref="B53" r:id="rId44" display="https://www.tinymachines3d.com/products/bigtreetech-tmc2209-v1-3"/>
-    <hyperlink ref="B56" r:id="rId45" display="DigiKey, Mouser, McMaster, Thorlabs and Amazon product pages could not be loaded from this environment; JLCPCB cannot quote without file upload."/>
+    <hyperlink ref="B18" r:id="rId10" display="https://jlcpcb.com/"/>
+    <hyperlink ref="B19" r:id="rId11" display="https://www.digikey.com/en/products/detail/analog-devices-inc/LT1469IN8-PBF/962892"/>
+    <hyperlink ref="B20" r:id="rId12" display="https://www.digikey.com/en/products/detail/ohmite/SM104031007FE/824190"/>
+    <hyperlink ref="B21" r:id="rId13" display="https://octopart.com/part/keystone/11301"/>
+    <hyperlink ref="B22" r:id="rId14" display="https://www.lcsc.com/product-detail/C50636.html"/>
+    <hyperlink ref="B24" r:id="rId15" display="https://www.jameco.com/z/182M18-Hammond-Manufacturing-Toroidal-Transformer-120VA-50Hz-Dual-Secondary-36VCT-3-33A-Series-18V-6-66A-Parallel_2575671.html"/>
+    <hyperlink ref="B25" r:id="rId16" display="https://batteryjunction.com/batteries/shop-by-size/9v/energizer-522bp-4"/>
+    <hyperlink ref="B26" r:id="rId17" display="https://octopart.com/part/keystone/1294"/>
+    <hyperlink ref="B27" r:id="rId18" display="https://www.sparkfun.com/teensy-4-1.html"/>
+    <hyperlink ref="B28" r:id="rId19" display="https://adafruit.com/product/4821"/>
+    <hyperlink ref="B29" r:id="rId20" display="https://store.sunlu.com/products/petg-cfpetg-carbon-fiber-3d-printer-filament-1kg"/>
+    <hyperlink ref="B30" r:id="rId21" display="https://www.walmart.com/ip/533082272"/>
+    <hyperlink ref="B31" r:id="rId22" display="https://www.tedpella.com/AFM_html/AFM.aspx"/>
+    <hyperlink ref="B32" r:id="rId23" display="https://www.isolateit.com/products/sorbothane-acoustic-and-vibration-isolation-square-6-x-6-pads"/>
+    <hyperlink ref="B33" r:id="rId24" display="https://jlc3dp.com/help/article/us-tariff-policy-faq"/>
+    <hyperlink ref="B34" r:id="rId25" display="https://www.piezodrive.com/?p=991"/>
+    <hyperlink ref="B35" r:id="rId26" display="https://www.piezodrive.com/piezoelectric-tube-scanners/"/>
+    <hyperlink ref="B36" r:id="rId27" display="https://www.piezodrive.com/product-category/tube-scanners/"/>
+    <hyperlink ref="B37" r:id="rId28" display="https://www.piezodrive.com/product/pdu150-three-channel-ultra-low-noise-150v-piezo-driver/"/>
+    <hyperlink ref="B38" r:id="rId29" display="https://www.piezodrive.com/product/ps1-24v-power-supply-for-modules/"/>
+    <hyperlink ref="B39" r:id="rId30" display="https://www.piezodrive.com/product/td250-six-channel-250v/"/>
+    <hyperlink ref="B40" r:id="rId31" display="https://www.piezodrive.com/product/horizontal-tube-wiring/"/>
+    <hyperlink ref="B41" r:id="rId32" display="https://trykintsugi.com/sales-tax-guides/usa/california/san-diego-county.md"/>
+    <hyperlink ref="B42" r:id="rId33" display="https://www.eevblog.com/forum/manufacture/lcscglobal-direct-shipping-to-usa-tariff-question/"/>
+    <hyperlink ref="B43" r:id="rId34" display="https://mae156b.eng.ucsd.edu/mae156-resources/mae-undergrad-lab-resources/lab-shops/ucsd-lab-shop-resources-outside-of-mae"/>
+    <hyperlink ref="B44" r:id="rId35" display="https://mpl.ucsd.edu/machine-shop-info/"/>
+    <hyperlink ref="B45" r:id="rId36" display="https://jacobsschool.ucsd.edu/envision"/>
+    <hyperlink ref="B46" r:id="rId37" display="https://www.goodfellow.com/usa/macor-glass-ceramic-rod-1000004916"/>
+    <hyperlink ref="B47" r:id="rId38" display="https://store.bruker.com/products/dpt10"/>
+    <hyperlink ref="B48" r:id="rId39" display="https://www.2spi.com/item/z01707/"/>
+    <hyperlink ref="B49" r:id="rId40" display="https://www.sigmaaldrich.com/US/en/product/aldrich/gf84004523"/>
+    <hyperlink ref="B50" r:id="rId41" display="https://www.penntoolco.com/grizzly-12-x-18-x-3-granite-surface-plate-no-ledge-g9651"/>
+    <hyperlink ref="B51" r:id="rId42" display="https://www.batterymart.com/p-energizer-la522-9volt-lithium-battery.html"/>
+    <hyperlink ref="B52" r:id="rId43" display="https://vetco.net/products/8331d-14g_silver_conductive_epoxy_adhesive_-_mg_chemicals_8331d-14g"/>
+    <hyperlink ref="B53" r:id="rId44" display="https://kozakmicro.com/collections/1-4-80-tpi-oem-alternative-screws"/>
+    <hyperlink ref="B54" r:id="rId45" display="https://www.tinymachines3d.com/products/bigtreetech-tmc2209-v1-3"/>
+    <hyperlink ref="B57" r:id="rId46" display="DigiKey, Mouser, McMaster, Thorlabs and Amazon product pages could not be loaded from this environment; JLCPCB cannot quote without file upload."/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3183,7 +3210,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3446,180 +3473,180 @@
         <v>3</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>8.78</v>
+        <v>8.8</v>
       </c>
       <c r="K10" s="3" t="n">
         <f aca="false">I10*J10</f>
-        <v>26.34</v>
+        <v>26.4</v>
       </c>
       <c r="L10" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="M10" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="M10" s="7" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="B11" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I11" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <f aca="false">I11*J11</f>
+        <v>25.8</v>
+      </c>
+      <c r="L11" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="14"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="14"/>
-    </row>
-    <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="F12" s="16" t="s">
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+    </row>
+    <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
         <v>89</v>
-      </c>
-      <c r="G12" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="I12" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" s="3" t="n">
-        <v>209.64</v>
-      </c>
-      <c r="K12" s="3" t="n">
-        <f aca="false">I12*J12</f>
-        <v>419.28</v>
-      </c>
-      <c r="L12" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="M12" s="7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>92</v>
       </c>
       <c r="B13" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F13" s="16" t="s">
         <v>93</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>89</v>
       </c>
       <c r="G13" s="0" t="n">
         <v>2</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="I13" s="0" t="n">
         <v>2</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>30.17</v>
+        <v>209.64</v>
       </c>
       <c r="K13" s="3" t="n">
         <f aca="false">I13*J13</f>
-        <v>60.34</v>
+        <v>419.28</v>
       </c>
       <c r="L13" s="15" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B14" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G14" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>64</v>
+        <v>94</v>
       </c>
       <c r="I14" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>1.68</v>
+        <v>30.17</v>
       </c>
       <c r="K14" s="3" t="n">
         <f aca="false">I14*J14</f>
-        <v>5.04</v>
+        <v>60.34</v>
       </c>
       <c r="L14" s="15" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B15" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G15" s="0" t="n">
         <v>3</v>
@@ -3631,141 +3658,141 @@
         <v>3</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.8</v>
+        <v>1.68</v>
       </c>
       <c r="K15" s="3" t="n">
         <f aca="false">I15*J15</f>
-        <v>2.4</v>
+        <v>5.04</v>
       </c>
       <c r="L15" s="15" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>104</v>
-      </c>
       <c r="E16" s="15" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G16" s="0" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
       <c r="I16" s="0" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="K16" s="3" t="n">
         <f aca="false">I16*J16</f>
+        <v>2.4</v>
+      </c>
+      <c r="L16" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="I17" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <f aca="false">I17*J17</f>
         <v>10</v>
       </c>
-      <c r="L16" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="M16" s="7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="L17" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-    </row>
-    <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="B18" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="E18" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="F18" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="G18" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="I18" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="J18" s="3" t="n">
-        <v>18.26</v>
-      </c>
-      <c r="K18" s="3" t="n">
-        <f aca="false">I18*J18</f>
-        <v>36.52</v>
-      </c>
-      <c r="L18" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="M18" s="7" t="s">
-        <v>113</v>
-      </c>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
+      <c r="J18" s="14"/>
+      <c r="K18" s="14"/>
+      <c r="L18" s="14"/>
+      <c r="M18" s="14"/>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B19" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C19" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="15" t="s">
         <v>116</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>111</v>
       </c>
       <c r="F19" s="16" t="s">
         <v>117</v>
       </c>
       <c r="G19" s="0" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>64</v>
@@ -3774,37 +3801,37 @@
         <v>2</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>5.73</v>
+        <v>18.26</v>
       </c>
       <c r="K19" s="3" t="n">
         <f aca="false">I19*J19</f>
-        <v>11.46</v>
+        <v>36.52</v>
       </c>
       <c r="L19" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="M19" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="M19" s="7" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B20" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C20" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="E20" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="F20" s="16" t="s">
         <v>122</v>
-      </c>
-      <c r="E20" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>123</v>
       </c>
       <c r="G20" s="0" t="n">
         <v>1</v>
@@ -3816,14 +3843,14 @@
         <v>2</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>2.09</v>
+        <v>5.73</v>
       </c>
       <c r="K20" s="3" t="n">
         <f aca="false">I20*J20</f>
-        <v>4.18</v>
+        <v>11.46</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>124</v>
@@ -3843,312 +3870,312 @@
         <v>127</v>
       </c>
       <c r="E21" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="F21" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="F21" s="16" t="s">
-        <v>129</v>
-      </c>
       <c r="G21" s="0" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>64</v>
       </c>
       <c r="I21" s="0" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>6.7247</v>
+        <v>2.09</v>
       </c>
       <c r="K21" s="3" t="n">
         <f aca="false">I21*J21</f>
-        <v>40.3482</v>
+        <v>4.18</v>
       </c>
       <c r="L21" s="15" t="s">
-        <v>65</v>
+        <v>95</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B22" s="0" t="s">
         <v>9</v>
       </c>
       <c r="C22" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="E22" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="E22" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="16" t="s">
         <v>134</v>
       </c>
       <c r="G22" s="0" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H22" s="15" t="s">
-        <v>135</v>
+        <v>64</v>
       </c>
       <c r="I22" s="0" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>40</v>
+        <v>6.7247</v>
       </c>
       <c r="K22" s="3" t="n">
         <f aca="false">I22*J22</f>
+        <v>40.3482</v>
+      </c>
+      <c r="L22" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="M22" s="7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="B23" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="G23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="I23" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="L22" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="M22" s="7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="K23" s="3" t="n">
+        <f aca="false">I23*J23</f>
+        <v>40</v>
+      </c>
+      <c r="L23" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="M23" s="7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="J23" s="14"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
-      <c r="M23" s="14"/>
-    </row>
-    <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
-        <v>137</v>
-      </c>
-      <c r="B24" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="F24" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="G24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="I24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="3" t="n">
-        <v>67.85</v>
-      </c>
-      <c r="K24" s="3" t="n">
-        <f aca="false">I24*J24</f>
-        <v>67.85</v>
-      </c>
-      <c r="L24" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="M24" s="7" t="s">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="14"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="14"/>
+      <c r="L24" s="14"/>
+      <c r="M24" s="14"/>
+    </row>
+    <row r="25" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
-        <v>143</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>10</v>
       </c>
       <c r="C25" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="E25" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="F25" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="F25" s="16" t="s">
-        <v>147</v>
-      </c>
       <c r="G25" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>148</v>
+        <v>64</v>
       </c>
       <c r="I25" s="0" t="n">
         <v>1</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>20.85</v>
+        <v>67.85</v>
       </c>
       <c r="K25" s="3" t="n">
         <f aca="false">I25*J25</f>
-        <v>20.85</v>
+        <v>67.85</v>
       </c>
       <c r="L25" s="15" t="s">
-        <v>65</v>
+        <v>111</v>
       </c>
       <c r="M25" s="7" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B26" s="0" t="s">
         <v>10</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E26" s="15" t="s">
         <v>151</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="F26" s="16" t="s">
         <v>152</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="F26" s="16" t="s">
-        <v>153</v>
       </c>
       <c r="G26" s="0" t="n">
         <v>2</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>64</v>
+        <v>153</v>
       </c>
       <c r="I26" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>2.99</v>
+        <v>20.85</v>
       </c>
       <c r="K26" s="3" t="n">
         <f aca="false">I26*J26</f>
-        <v>5.98</v>
+        <v>20.85</v>
       </c>
       <c r="L26" s="15" t="s">
-        <v>118</v>
+        <v>65</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+    <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="F27" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="G27" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I27" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="K27" s="3" t="n">
+        <f aca="false">I27*J27</f>
+        <v>5.98</v>
+      </c>
+      <c r="L27" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="M27" s="7" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="14"/>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
-        <v>155</v>
-      </c>
-      <c r="B28" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="D28" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>158</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="G28" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="H28" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="I28" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J28" s="3" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="K28" s="3" t="n">
-        <f aca="false">I28*J28</f>
-        <v>31.5</v>
-      </c>
-      <c r="L28" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="M28" s="7" t="s">
+      <c r="B28" s="14"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="14"/>
+      <c r="L28" s="14"/>
+      <c r="M28" s="14"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
-        <v>161</v>
       </c>
       <c r="B29" s="0" t="s">
         <v>11</v>
       </c>
       <c r="C29" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="E29" s="15" t="s">
         <v>163</v>
-      </c>
-      <c r="E29" s="15" t="s">
-        <v>70</v>
       </c>
       <c r="F29" s="16" t="s">
         <v>164</v>
       </c>
       <c r="G29" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>64</v>
       </c>
       <c r="I29" s="0" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>11.5</v>
+        <v>31.5</v>
       </c>
       <c r="K29" s="3" t="n">
         <f aca="false">I29*J29</f>
-        <v>23</v>
+        <v>31.5</v>
       </c>
       <c r="L29" s="15" t="s">
         <v>65</v>
@@ -4157,203 +4184,245 @@
         <v>165</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+    <row r="30" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="G30" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="I30" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <f aca="false">I30*J30</f>
+        <v>23</v>
+      </c>
+      <c r="L30" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="M30" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="14"/>
-      <c r="G30" s="14"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="14"/>
-      <c r="J30" s="14"/>
-      <c r="K30" s="14"/>
-      <c r="L30" s="14"/>
-      <c r="M30" s="14"/>
-    </row>
-    <row r="31" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="E31" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="F31" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="G31" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="H31" s="15" t="s">
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
+      <c r="M31" s="14"/>
+    </row>
+    <row r="32" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
         <v>171</v>
-      </c>
-      <c r="I31" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" s="3" t="n">
-        <v>19.99</v>
-      </c>
-      <c r="K31" s="3" t="n">
-        <f aca="false">I31*J31</f>
-        <v>19.99</v>
-      </c>
-      <c r="L31" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="M31" s="7" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
-        <v>173</v>
       </c>
       <c r="B32" s="0" t="s">
         <v>12</v>
       </c>
       <c r="C32" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="E32" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="F32" s="16" t="s">
         <v>175</v>
       </c>
-      <c r="E32" s="15" t="s">
+      <c r="G32" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="15" t="s">
         <v>176</v>
-      </c>
-      <c r="F32" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="G32" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="15" t="s">
-        <v>178</v>
       </c>
       <c r="I32" s="0" t="n">
         <v>1</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>9.99</v>
+        <v>19.99</v>
       </c>
       <c r="K32" s="3" t="n">
         <f aca="false">I32*J32</f>
-        <v>9.99</v>
+        <v>19.99</v>
       </c>
       <c r="L32" s="15" t="s">
         <v>65</v>
       </c>
       <c r="M32" s="7" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B33" s="0" t="s">
         <v>12</v>
       </c>
       <c r="C33" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="E33" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="F33" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="E33" s="15" t="s">
+      <c r="G33" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H33" s="15" t="s">
         <v>183</v>
-      </c>
-      <c r="F33" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="G33" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" s="15" t="s">
-        <v>185</v>
       </c>
       <c r="I33" s="0" t="n">
         <v>1</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>30</v>
+        <v>9.99</v>
       </c>
       <c r="K33" s="3" t="n">
         <f aca="false">I33*J33</f>
-        <v>30</v>
+        <v>9.99</v>
       </c>
       <c r="L33" s="15" t="s">
         <v>65</v>
       </c>
       <c r="M33" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B34" s="0" t="s">
         <v>12</v>
       </c>
       <c r="C34" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="E34" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="F34" s="16" t="s">
         <v>189</v>
       </c>
-      <c r="E34" s="15" t="s">
+      <c r="G34" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" s="15" t="s">
         <v>190</v>
-      </c>
-      <c r="F34" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="G34" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="H34" s="15" t="s">
-        <v>192</v>
       </c>
       <c r="I34" s="0" t="n">
         <v>1</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="K34" s="3" t="n">
         <f aca="false">I34*J34</f>
+        <v>30</v>
+      </c>
+      <c r="L34" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="M34" s="7" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>192</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="F35" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="G35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="I35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="3" t="n">
         <v>35</v>
       </c>
-      <c r="L34" s="15" t="s">
-        <v>106</v>
-      </c>
-      <c r="M34" s="7" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="K35" s="3" t="n">
+        <f aca="false">I35*J35</f>
+        <v>35</v>
+      </c>
+      <c r="L35" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="M35" s="7" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="0" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C36" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="K36" s="12" t="n">
-        <f aca="false">SUM(K5:K34)</f>
-        <v>1054.0182</v>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C37" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="K37" s="12" t="n">
+        <f aca="false">SUM(K5:K35)</f>
+        <v>1079.8782</v>
       </c>
     </row>
   </sheetData>
@@ -4362,24 +4431,25 @@
     <hyperlink ref="F8" r:id="rId2" display="https://www.adafruit.com/product/324"/>
     <hyperlink ref="F9" r:id="rId3" display="https://adafruit.com/product/6121"/>
     <hyperlink ref="F10" r:id="rId4" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=FAS200"/>
-    <hyperlink ref="F12" r:id="rId5" display="https://jlcpcb.com/"/>
+    <hyperlink ref="F11" r:id="rId5" display="https://www.thorlabs.com/thorproduct.cfm?partnumber=F25SSN1"/>
     <hyperlink ref="F13" r:id="rId6" display="https://jlcpcb.com/"/>
     <hyperlink ref="F14" r:id="rId7" display="https://jlcpcb.com/"/>
     <hyperlink ref="F15" r:id="rId8" display="https://jlcpcb.com/"/>
     <hyperlink ref="F16" r:id="rId9" display="https://jlcpcb.com/"/>
-    <hyperlink ref="F18" r:id="rId10" display="https://www.digikey.com/en/products/detail/analog-devices-inc/LT1469IN8-PBF/962892"/>
-    <hyperlink ref="F19" r:id="rId11" display="https://www.digikey.com/en/products/detail/ohmite/SM104031007FE/824190"/>
-    <hyperlink ref="F20" r:id="rId12" display="https://octopart.com/part/keystone/11301"/>
-    <hyperlink ref="F21" r:id="rId13" display="https://www.lcsc.com/product-detail/C50636.html"/>
-    <hyperlink ref="F24" r:id="rId14" display="https://www.jameco.com/z/182M18-Hammond-Manufacturing-Toroidal-Transformer-120VA-50Hz-Dual-Secondary-36VCT-3-33A-Series-18V-6-66A-Parallel_2575671.html"/>
-    <hyperlink ref="F25" r:id="rId15" display="https://batteryjunction.com/batteries/shop-by-size/9v/energizer-522bp-4"/>
-    <hyperlink ref="F26" r:id="rId16" display="https://octopart.com/part/keystone/1294"/>
-    <hyperlink ref="F28" r:id="rId17" display="https://www.sparkfun.com/teensy-4-1.html"/>
-    <hyperlink ref="F29" r:id="rId18" display="https://adafruit.com/product/4821"/>
-    <hyperlink ref="F31" r:id="rId19" display="https://store.sunlu.com/products/petg-cfpetg-carbon-fiber-3d-printer-filament-1kg"/>
-    <hyperlink ref="F32" r:id="rId20" display="https://www.walmart.com/ip/533082272"/>
-    <hyperlink ref="F33" r:id="rId21" display="https://www.tedpella.com/AFM_html/AFM.aspx"/>
-    <hyperlink ref="F34" r:id="rId22" display="https://www.isolateit.com/products/sorbothane-acoustic-and-vibration-isolation-square-6-x-6-pads"/>
+    <hyperlink ref="F17" r:id="rId10" display="https://jlcpcb.com/"/>
+    <hyperlink ref="F19" r:id="rId11" display="https://www.digikey.com/en/products/detail/analog-devices-inc/LT1469IN8-PBF/962892"/>
+    <hyperlink ref="F20" r:id="rId12" display="https://www.digikey.com/en/products/detail/ohmite/SM104031007FE/824190"/>
+    <hyperlink ref="F21" r:id="rId13" display="https://octopart.com/part/keystone/11301"/>
+    <hyperlink ref="F22" r:id="rId14" display="https://www.lcsc.com/product-detail/C50636.html"/>
+    <hyperlink ref="F25" r:id="rId15" display="https://www.jameco.com/z/182M18-Hammond-Manufacturing-Toroidal-Transformer-120VA-50Hz-Dual-Secondary-36VCT-3-33A-Series-18V-6-66A-Parallel_2575671.html"/>
+    <hyperlink ref="F26" r:id="rId16" display="https://batteryjunction.com/batteries/shop-by-size/9v/energizer-522bp-4"/>
+    <hyperlink ref="F27" r:id="rId17" display="https://octopart.com/part/keystone/1294"/>
+    <hyperlink ref="F29" r:id="rId18" display="https://www.sparkfun.com/teensy-4-1.html"/>
+    <hyperlink ref="F30" r:id="rId19" display="https://adafruit.com/product/4821"/>
+    <hyperlink ref="F32" r:id="rId20" display="https://store.sunlu.com/products/petg-cfpetg-carbon-fiber-3d-printer-filament-1kg"/>
+    <hyperlink ref="F33" r:id="rId21" display="https://www.walmart.com/ip/533082272"/>
+    <hyperlink ref="F34" r:id="rId22" display="https://www.tedpella.com/AFM_html/AFM.aspx"/>
+    <hyperlink ref="F35" r:id="rId23" display="https://www.isolateit.com/products/sorbothane-acoustic-and-vibration-isolation-square-6-x-6-pads"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4412,12 +4482,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4430,31 +4500,31 @@
         <v>51</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4462,17 +4532,17 @@
         <v>62</v>
       </c>
       <c r="B5" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A5,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A5,'Detailed BOM'!$K$5:$K$35)</f>
         <v>131</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>60</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="F5" s="17" t="n">
         <v>0.1</v>
@@ -4482,7 +4552,7 @@
         <v>13.1</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="I5" s="3" t="n">
         <f aca="false">B5*Assumptions!$B$5</f>
@@ -4498,14 +4568,14 @@
         <v>70</v>
       </c>
       <c r="B6" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A6,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A6,'Detailed BOM'!$K$5:$K$35)</f>
         <v>45.95</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>6</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F6" s="17" t="n">
         <v>0</v>
@@ -4528,17 +4598,17 @@
         <v>81</v>
       </c>
       <c r="B7" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A7,'Detailed BOM'!$K$5:$K$34)</f>
-        <v>26.34</v>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A7,'Detailed BOM'!$K$5:$K$35)</f>
+        <v>52.2</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>15.26</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="F7" s="17" t="n">
         <v>0</v>
@@ -4548,33 +4618,33 @@
         <v>0</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="I7" s="3" t="n">
         <f aca="false">B7*Assumptions!$B$5</f>
-        <v>2.04135</v>
+        <v>4.0455</v>
       </c>
       <c r="J7" s="3" t="n">
         <f aca="false">B7+C7+G7+I7</f>
-        <v>43.64135</v>
+        <v>71.5055</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A8,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A8,'Detailed BOM'!$K$5:$K$35)</f>
         <v>497.06</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>50.3</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="F8" s="17" t="n">
         <v>0.35</v>
@@ -4584,7 +4654,7 @@
         <v>173.971</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="I8" s="3" t="n">
         <f aca="false">B8*Assumptions!$B$5</f>
@@ -4597,20 +4667,20 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B9" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A9,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A9,'Detailed BOM'!$K$5:$K$35)</f>
         <v>58.14</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>8.49</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="F9" s="17" t="n">
         <v>0.08</v>
@@ -4620,7 +4690,7 @@
         <v>4.6512</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="I9" s="3" t="n">
         <f aca="false">B9*Assumptions!$B$5</f>
@@ -4633,20 +4703,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B10" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A10,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A10,'Detailed BOM'!$K$5:$K$35)</f>
         <v>80.3482</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>22.21</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="F10" s="17" t="n">
         <v>0.35</v>
@@ -4656,7 +4726,7 @@
         <v>28.12187</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="I10" s="3" t="n">
         <f aca="false">B10*Assumptions!$B$5</f>
@@ -4669,17 +4739,17 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B11" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A11,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A11,'Detailed BOM'!$K$5:$K$35)</f>
         <v>67.85</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F11" s="17" t="n">
         <v>0</v>
@@ -4699,17 +4769,17 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="B12" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A12,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A12,'Detailed BOM'!$K$5:$K$35)</f>
         <v>20.85</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>6</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F12" s="17" t="n">
         <v>0</v>
@@ -4729,17 +4799,17 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B13" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A13,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A13,'Detailed BOM'!$K$5:$K$35)</f>
         <v>31.5</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F13" s="17" t="n">
         <v>0</v>
@@ -4759,20 +4829,20 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B14" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A14,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A14,'Detailed BOM'!$K$5:$K$35)</f>
         <v>19.99</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="F14" s="17" t="n">
         <v>0</v>
@@ -4792,17 +4862,17 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B15" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A15,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A15,'Detailed BOM'!$K$5:$K$35)</f>
         <v>9.99</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F15" s="17" t="n">
         <v>0</v>
@@ -4822,17 +4892,17 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="B16" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A16,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A16,'Detailed BOM'!$K$5:$K$35)</f>
         <v>30</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>12</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F16" s="17" t="n">
         <v>0</v>
@@ -4852,17 +4922,17 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B17" s="3" t="n">
-        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$34,A17,'Detailed BOM'!$K$5:$K$34)</f>
+        <f aca="false">SUMIF('Detailed BOM'!$E$5:$E$35,A17,'Detailed BOM'!$K$5:$K$35)</f>
         <v>35</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="F17" s="17" t="n">
         <v>0</v>
@@ -4882,7 +4952,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B18" s="0" t="n">
         <v>0</v>
@@ -4891,13 +4961,13 @@
         <v>0</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G18" s="0" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="I18" s="0" t="n">
         <v>0</v>
@@ -4914,11 +4984,11 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B20" s="9" t="n">
         <f aca="false">SUM(B5:B17)</f>
-        <v>1054.0182</v>
+        <v>1079.8782</v>
       </c>
       <c r="C20" s="9" t="n">
         <f aca="false">SUM(C5:C17)</f>
@@ -4934,11 +5004,11 @@
       <c r="H20" s="8"/>
       <c r="I20" s="9" t="n">
         <f aca="false">SUM(I5:I17)</f>
-        <v>81.6864105</v>
+        <v>83.6905605</v>
       </c>
       <c r="J20" s="9" t="n">
         <f aca="false">SUM(J5:J18)</f>
-        <v>1624.8086805</v>
+        <v>1652.6728305</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4948,14 +5018,14 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="B22" s="3" t="n">
-        <f aca="false">B20-'Detailed BOM'!K36</f>
+        <f aca="false">B20-'Detailed BOM'!K37</f>
         <v>0</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -4986,12 +5056,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5001,198 +5071,198 @@
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>277.2</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>77</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>75.15</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>133.13</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -5235,12 +5305,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5250,37 +5320,37 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>5</v>
@@ -5288,22 +5358,22 @@
     </row>
     <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>131</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="F5" s="3" t="n">
-        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-01",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-02",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-03",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-04",'Detailed BOM'!$A$5:$A$34,0))</f>
+        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-01",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-02",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-03",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-04",'Detailed BOM'!$A$5:$A$35,0))</f>
         <v>158.1982</v>
       </c>
       <c r="G5" s="3" t="n">
@@ -5318,30 +5388,30 @@
         <v>0</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>288</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>289</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>283</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>284</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>278</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>131</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>892</v>
@@ -5358,30 +5428,30 @@
         <v>733.8018</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>131</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>3172</v>
@@ -5398,33 +5468,33 @@
         <v>3013.8018</v>
       </c>
       <c r="J7" s="15" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>111</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F8" s="3" t="n">
-        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-01",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-02",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-03",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-04",'Detailed BOM'!$A$5:$A$34,0))</f>
+        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-01",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-02",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-03",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-04",'Detailed BOM'!$A$5:$A$35,0))</f>
         <v>158.1982</v>
       </c>
       <c r="G8" s="3" t="n">
@@ -5439,33 +5509,33 @@
         <v>-20</v>
       </c>
       <c r="J8" s="15" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="K8" s="15" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>156</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F9" s="3" t="n">
-        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-01",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-02",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-03",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-04",'Detailed BOM'!$A$5:$A$34,0))</f>
+        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-01",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-02",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-03",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-04",'Detailed BOM'!$A$5:$A$35,0))</f>
         <v>158.1982</v>
       </c>
       <c r="G9" s="3" t="n">
@@ -5480,33 +5550,33 @@
         <v>25</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="K9" s="15" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>131</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="F10" s="3" t="n">
-        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-01",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-02",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-03",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("HV-04",'Detailed BOM'!$A$5:$A$34,0))</f>
+        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-01",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-02",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-03",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("HV-04",'Detailed BOM'!$A$5:$A$35,0))</f>
         <v>158.1982</v>
       </c>
       <c r="G10" s="3" t="n">
@@ -5521,13 +5591,13 @@
         <v>100</v>
       </c>
       <c r="J10" s="15" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="K10" s="15" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>
@@ -5561,12 +5631,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5576,21 +5646,21 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B4" s="3" t="n">
-        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$34,MATCH("PZ-02",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("PZ-03",'Detailed BOM'!$A$5:$A$34,0))+INDEX('Detailed BOM'!$K$5:$K$34,MATCH("PZ-04",'Detailed BOM'!$A$5:$A$34,0))</f>
-        <v>49.29</v>
+        <f aca="false">INDEX('Detailed BOM'!$K$5:$K$35,MATCH("PZ-02",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("PZ-03",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("PZ-04",'Detailed BOM'!$A$5:$A$35,0))+INDEX('Detailed BOM'!$K$5:$K$35,MATCH("PZ-05",'Detailed BOM'!$A$5:$A$35,0))</f>
+        <v>75.15</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5600,30 +5670,30 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="E9" s="19" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="H9" s="19" t="s">
         <v>5</v>
@@ -5631,13 +5701,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D10" s="0" t="n">
         <v>1</v>
@@ -5653,18 +5723,18 @@
         <v>65</v>
       </c>
       <c r="H10" s="15" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D11" s="0" t="n">
         <v>3</v>
@@ -5682,13 +5752,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D12" s="0" t="n">
         <v>1</v>
@@ -5706,20 +5776,20 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="F13" s="3" t="n">
-        <f aca="false">SUM(F10:F12)+INDEX('Detailed BOM'!$J$5:$J$34,MATCH("HV-01",'Detailed BOM'!$A$5:$A$34,0))</f>
+        <f aca="false">SUM(F10:F12)+INDEX('Detailed BOM'!$J$5:$J$35,MATCH("HV-01",'Detailed BOM'!$A$5:$A$35,0))</f>
         <v>164.2947</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="F14" s="3" t="n">
         <f aca="false">F13-B4</f>
-        <v>115.0047</v>
+        <v>89.1447</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5729,7 +5799,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>
@@ -5771,12 +5841,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5786,63 +5856,63 @@
     </row>
     <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E5" s="0" t="n">
         <v>3</v>
@@ -5878,24 +5948,24 @@
         <v>2.44913335386511</v>
       </c>
       <c r="N5" s="15" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="O5" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E6" s="0" t="n">
         <v>3</v>
@@ -5931,24 +6001,24 @@
         <v>1.166253978031</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="O6" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E7" s="0" t="n">
         <v>2</v>
@@ -5984,24 +6054,24 @@
         <v>305.609565855662</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="O7" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E8" s="0" t="n">
         <v>2</v>
@@ -6037,10 +6107,10 @@
         <v>43.9823531464942</v>
       </c>
       <c r="N8" s="15" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="O8" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6048,10 +6118,10 @@
         <v>81</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="D9" s="0" t="s">
         <v>80</v>
@@ -6090,24 +6160,24 @@
         <v>14.4166666666667</v>
       </c>
       <c r="N9" s="15" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="O9" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="E10" s="0" t="n">
         <v>2</v>
@@ -6142,24 +6212,24 @@
         <v>22.6647285954113</v>
       </c>
       <c r="N10" s="15" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="O10" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="E11" s="0" t="n">
         <v>4</v>
@@ -6194,24 +6264,24 @@
         <v>1.20513570229435</v>
       </c>
       <c r="N11" s="15" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="O11" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="E12" s="0" t="n">
         <v>2</v>
@@ -6246,24 +6316,24 @@
         <v>7.47</v>
       </c>
       <c r="N12" s="15" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="O12" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="E13" s="0" t="n">
         <v>2</v>
@@ -6298,15 +6368,15 @@
         <v>6.865</v>
       </c>
       <c r="N13" s="15" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="O13" s="15" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="G14" s="3" t="n">
         <f aca="false">SUM(G5:G13)</f>
@@ -6319,14 +6389,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="L15" s="3" t="n">
         <f aca="false">L14-832.1</f>
         <v>0</v>
       </c>
       <c r="M15" s="15" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6336,12 +6406,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>543.83</v>
@@ -6349,7 +6419,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="G19" s="3" t="n">
         <f aca="false">L14+G18</f>
@@ -6384,7 +6454,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6394,291 +6464,291 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>402</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>404</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>397</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>399</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
+        <v>434</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>435</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>429</v>
       </c>
-      <c r="B17" s="7" t="s">
-        <v>430</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>424</v>
-      </c>
       <c r="D17" s="7" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -6709,12 +6779,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6724,80 +6794,80 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>0.0775</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>0.1</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>65</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>105</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>2000</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6807,27 +6877,27 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="7" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="7" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="7" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="7" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6837,187 +6907,187 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>504</v>
+        <v>509</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>505</v>
+        <v>510</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>506</v>
+        <v>511</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>507</v>
+        <v>512</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>508</v>
+        <v>513</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>509</v>
+        <v>514</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>510</v>
+        <v>515</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>511</v>
+        <v>516</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>512</v>
+        <v>517</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>513</v>
+        <v>518</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>514</v>
+        <v>519</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>515</v>
+        <v>520</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>516</v>
+        <v>521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v2 budget: add piezo tube mount and wiring, OPA454 6 to 5, LCR meter and interferometer parts
Totals now $2,994.45 if UCSD supplies nothing, $1,936.90 if it supplies everything.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1g5ouZCd4fvcL4KzTMSdf
</commit_message>
<xml_diff>
--- a/docs/v2-budget/STM_v2_budget.xlsx
+++ b/docs/v2-budget/STM_v2_budget.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="294">
   <si>
     <t xml:space="preserve">STM v1: what it actually cost</t>
   </si>
@@ -176,19 +176,19 @@
     <t xml:space="preserve">STM v2 at UCSD: budget</t>
   </si>
   <si>
-    <t xml:space="preserve">What this is: a scanning tunneling microscope (STM) images individual atoms by holding a sharp metal tip a few atoms above a sample and measuring the tiny electric current that flows across the gap. This sheet lists everything needed to build a second one (v2) at UCSD. Prices checked 21 October 2026, in US dollars. Sections 1 to 8 are parts we must buy. The microscope runs entirely on batteries (section 8), with no wall power. Section 9 lists items UCSD labs may already have; with nothing marked, the total assumes we buy all of them, which is why it starts above $2,000.</t>
+    <t xml:space="preserve">What this is: a scanning tunneling microscope (STM) images individual atoms by holding a sharp metal tip a few atoms above a sample and measuring the tiny electric current that flows across the gap. This sheet lists everything needed to build a second one (v2) at UCSD. Prices checked 21 October 2026, in US dollars. Sections 1 to 9 are parts we must buy. The microscope runs entirely on batteries (section 9), with no wall power. Section 10 lists items UCSD labs may already have; with nothing marked, the total assumes we buy all of them, which is why it starts above $2,000.</t>
   </si>
   <si>
     <t xml:space="preserve">Summary</t>
   </si>
   <si>
-    <t xml:space="preserve">Total request for v2 (updates as section 9 items are marked Yes)</t>
+    <t xml:space="preserve">Total request for v2 (updates as section 10 items are marked Yes)</t>
   </si>
   <si>
     <t xml:space="preserve">Room left under the $2,000 target</t>
   </si>
   <si>
-    <t xml:space="preserve">Total if UCSD supplies everything in section 9</t>
+    <t xml:space="preserve">Total if UCSD supplies everything in section 10</t>
   </si>
   <si>
     <t xml:space="preserve">What v1 actually cost, for comparison</t>
@@ -233,13 +233,136 @@
     <t xml:space="preserve">TB3006-N</t>
   </si>
   <si>
-    <t xml:space="preserve">2. High-voltage driver (powers the piezo tube)</t>
+    <t xml:space="preserve">2. Scanner mount and wiring (holds the tube and connects it)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceramic mounting block</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A small block of machinable ceramic that the tube is glued to. It holds the tube rigidly and insulates it electrically. Estimate; it needs a few holes drilled. If drilling is not possible, an aluminium block with an insulating epoxy layer is the fallback.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Needed to mount the tube.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Macor rod or plate offcut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Structural epoxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strong glue that bonds the tube to its mounting block. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. v1's parts were held with superglue, which gives off fumes that contaminate the electronics.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loctite EA E-30CL or similar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conductive silver epoxy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glue that conducts electricity. It attaches the wires to the tube's contacts without soldering heat, which can damage the tube. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Needed to wire the tube.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CW2400 or similar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tip holder tubing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short pieces of thin stainless steel tube that grip the scanning tip at the end of the piezo tube. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Replaces v1's glued tip holder.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stainless hypodermic tubing, about 23 gauge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thin shielded tip cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Very thin (about 1 mm) shielded cable that carries the tiny tip current to the preamp. 1 m. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. The tip now moves with the tube, so its cable must be thin and flexible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">micro-coax, about 1 mm, 1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-voltage box</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metal box that holds the high-voltage driver board (section 3), keeping the 45 V away from fingers and blocking electrical noise. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. The driver sits in its own box, between the main board and the microscope.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diecast aluminium, about 112 x 60 x 31 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9-pin connectors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plugs and sockets that connect the high-voltage box to the main board and to the microscope head. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Goes with the high-voltage box.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB9 plug and socket with covers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High-voltage cable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shielded cable with 5 wires, rated for at least 100 V, from the high-voltage box to the microscope head. 1 m. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Carries the 45 V signals to the tube.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5-core shielded cable, 1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test capacitors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small capacitors that stand in for the tube when the high-voltage box is first tested, so a wiring mistake cannot crack the tube. 4 plus 4 spares. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Protects the tube during testing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 nF 100 V film</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Threaded inserts and screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small metal inserts melted into the printed plate, with screws, to fix the mounting block to the head. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 heat-set inserts and screws</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. High-voltage driver (powers the piezo tube)</t>
   </si>
   <si>
     <t xml:space="preserve">Amplifier chips</t>
   </si>
   <si>
-    <t xml:space="preserve">The tube has 5 electrical contacts. Each needs its own amplifier chip to raise the control signal to about 45 V. 5 chips plus 1 spare. Powered by batteries (section 8).</t>
+    <t xml:space="preserve">The tube has 4 outer electrical contacts that move it; the inner one is simply connected to ground. Each outer contact needs its own amplifier chip to raise the control signal to about 45 V. 4 chips plus 1 spare. Powered by batteries (section 9).</t>
   </si>
   <si>
     <t xml:space="preserve">New. The tube needs far more voltage than v1's electronics can supply.</t>
@@ -275,13 +398,13 @@
     <t xml:space="preserve">custom</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Coarse approach (brings the sample close to the tip)</t>
+    <t xml:space="preserve">4. Coarse approach (brings the sample close to the tip)</t>
   </si>
   <si>
     <t xml:space="preserve">Motor</t>
   </si>
   <si>
-    <t xml:space="preserve">A motor that turns in small, precise steps. It slowly turns one adjustment screw to bring the sample up to the tip, then the piezo tube takes over. Joined to the screw by a 3D-printed coupler and powered by AA batteries (section 8).</t>
+    <t xml:space="preserve">A motor that turns in small, precise steps. It slowly turns one adjustment screw to bring the sample up to the tip, then the piezo tube takes over. Joined to the screw by a 3D-printed coupler and powered by AA batteries (section 9).</t>
   </si>
   <si>
     <t xml:space="preserve">New. Replaces v1's small toy-grade motor. Finer steps lower the risk of crashing the tip into the sample.</t>
@@ -296,7 +419,7 @@
     <t xml:space="preserve">Motor controller</t>
   </si>
   <si>
-    <t xml:space="preserve">A small board that lets the microcontroller (section 4) move the motor in tiny fractions of a step.</t>
+    <t xml:space="preserve">A small board that lets the microcontroller (section 5) move the motor in tiny fractions of a step.</t>
   </si>
   <si>
     <t xml:space="preserve">New. Needed to run the new motor.</t>
@@ -332,7 +455,7 @@
     <t xml:space="preserve">F25SSN1</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Control electronics (runs the microscope)</t>
+    <t xml:space="preserve">5. Control electronics (runs the microscope)</t>
   </si>
   <si>
     <t xml:space="preserve">Main circuit boards</t>
@@ -380,7 +503,7 @@
     <t xml:space="preserve">Teensy 4.1</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Preamp (amplifies the tiny tip current)</t>
+    <t xml:space="preserve">6. Preamp (amplifies the tiny tip current)</t>
   </si>
   <si>
     <t xml:space="preserve">Preamp circuit boards</t>
@@ -428,13 +551,10 @@
     <t xml:space="preserve">Same kind as v1. Listed here because general labs rarely stock it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Amazon</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kirecoo copper foil tape, 2 in x 33 ft</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Sample plate and frame</t>
+    <t xml:space="preserve">7. Sample plate and frame</t>
   </si>
   <si>
     <t xml:space="preserve">1 kg spool of carbon-fiber reinforced plastic for printing the head, sample plate and frame.</t>
@@ -500,7 +620,7 @@
     <t xml:space="preserve">Sorbothane 6x6 in, 2-pack</t>
   </si>
   <si>
-    <t xml:space="preserve">7. Sensors</t>
+    <t xml:space="preserve">8. Sensors</t>
   </si>
   <si>
     <t xml:space="preserve">Temperature sensors</t>
@@ -515,7 +635,7 @@
     <t xml:space="preserve">4821 (TMP117)</t>
   </si>
   <si>
-    <t xml:space="preserve">8. Power (batteries, no wall power)</t>
+    <t xml:space="preserve">9. Power (batteries, no wall power)</t>
   </si>
   <si>
     <t xml:space="preserve">9 V batteries</t>
@@ -572,13 +692,13 @@
     <t xml:space="preserve">All parts above</t>
   </si>
   <si>
-    <t xml:space="preserve">For sections 1 to 8 (section 9 prices do not include shipping). Estimates by seller: PiezoDrive $60.00, JLCPCB $25.00, Thorlabs $15.26, Ted Pella $15.00, Adafruit $10.00, Isolate It $10.00, Battery Junction $10.00, DigiKey $8.49, SparkFun $8.00, SUNLU $5.00. Amazon items ship free. Standard (not express) shipping everywhere, and the small electronic parts ship in the same box as the circuit boards.</t>
+    <t xml:space="preserve">For sections 1 to 9 (section 10 prices do not include shipping). Estimates by seller: PiezoDrive $60.00, JLCPCB $25.00, Thorlabs $15.26, Ted Pella $15.00, Adafruit $10.00, Isolate It $10.00, Battery Junction $10.00, DigiKey $8.49, SparkFun $8.00, SUNLU $5.00. Amazon items ship free. Standard (not express) shipping everywhere, and the small electronic parts ship in the same box as the circuit boards.</t>
   </si>
   <si>
     <t xml:space="preserve">Import tariff on circuit boards</t>
   </si>
   <si>
-    <t xml:space="preserve">The US charges a 35% import tariff on circuit boards and parts from China. Applied to the $577.41 of boards and parts from JLCPCB and LCSC. Cannot be avoided by changing shipping; only US-made boards would avoid it, and those cost more.</t>
+    <t xml:space="preserve">The US charges a 35% import tariff on circuit boards and parts from China. Applied to the $570.68 of boards and parts from JLCPCB and LCSC. Cannot be avoided by changing shipping; only US-made boards would avoid it, and those cost more.</t>
   </si>
   <si>
     <t xml:space="preserve">Other import fees</t>
@@ -593,7 +713,7 @@
     <t xml:space="preserve">UCSD purchasing may have its own shipping accounts or negotiated rates with these sellers, which could lower this. Not counted here.</t>
   </si>
   <si>
-    <t xml:space="preserve">9. Things UCSD may already have: choose Yes in the last column if UCSD will provide it, and it comes off the total</t>
+    <t xml:space="preserve">10. Things UCSD may already have: choose Yes in the last column if UCSD will provide it, and it comes off the total</t>
   </si>
   <si>
     <t xml:space="preserve">Free from UCSD?</t>
@@ -668,6 +788,30 @@
     <t xml:space="preserve">FNIRSI DST-201</t>
   </si>
   <si>
+    <t xml:space="preserve">LCR meter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A handheld meter that measures capacitance. Used to check each of the tube's contacts before and after wiring. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Confirms the tube was not damaged during assembly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">handheld LCR meter, 1 kHz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interferometer parts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A small laser, a beam splitter, two mirrors and a light sensor. Together they measure exactly how far the scanner moves per volt, which calibrates the images. Estimate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New. Calibrates the scanner.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">laser diode, beamsplitter cube, 2 mirrors, photodiode, mounts</t>
+  </si>
+  <si>
     <t xml:space="preserve">Soldering iron</t>
   </si>
   <si>
@@ -734,7 +878,7 @@
     <t xml:space="preserve">Parts</t>
   </si>
   <si>
-    <t xml:space="preserve">Sections 1 to 8, plus section 9 items not marked Yes</t>
+    <t xml:space="preserve">Sections 1 to 9, plus section 10 items not marked Yes</t>
   </si>
   <si>
     <t xml:space="preserve">Shipping and import fees</t>
@@ -758,10 +902,10 @@
     <t xml:space="preserve">For comparison</t>
   </si>
   <si>
-    <t xml:space="preserve">If UCSD provides everything in section 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If UCSD provides nothing in section 9</t>
+    <t xml:space="preserve">If UCSD provides everything in section 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If UCSD provides nothing in section 10</t>
   </si>
 </sst>
 </file>
@@ -1853,7 +1997,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J111"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -1898,8 +2042,8 @@
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="17" t="n">
-        <f aca="false">H91</f>
-        <v>2732.4</v>
+        <f aca="false">H106</f>
+        <v>2994.445</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1908,8 +2052,8 @@
       </c>
       <c r="B6" s="18"/>
       <c r="C6" s="19" t="n">
-        <f aca="false">H92</f>
-        <v>-732.4</v>
+        <f aca="false">H107</f>
+        <v>-994.445</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1918,8 +2062,8 @@
       </c>
       <c r="B7" s="18"/>
       <c r="C7" s="19" t="n">
-        <f aca="false">H95</f>
-        <v>1793.37</v>
+        <f aca="false">H110</f>
+        <v>1936.9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2034,7 +2178,7 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
     </row>
-    <row r="16" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
         <v>70</v>
       </c>
@@ -2051,17 +2195,17 @@
         <v>74</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G16" s="23" t="n">
-        <v>6.725</v>
+        <v>35</v>
       </c>
       <c r="H16" s="23" t="n">
         <f aca="false">F16*G16</f>
-        <v>40.35</v>
+        <v>35</v>
       </c>
       <c r="I16" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.lcsc.com/product-detail/C50636.html","Open")</f>
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=Macor+machinable+ceramic+rod","Open")</f>
         <v>Open</v>
       </c>
     </row>
@@ -2085,14 +2229,14 @@
         <v>1</v>
       </c>
       <c r="G17" s="23" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="H17" s="23" t="n">
         <f aca="false">F17*G17</f>
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="I17" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.lcsc.com/","Open")</f>
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=Loctite+EA+E-30CL+epoxy","Open")</f>
         <v>Open</v>
       </c>
     </row>
@@ -2104,179 +2248,243 @@
         <v>80</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E18" s="22" t="s">
         <v>82</v>
       </c>
       <c r="F18" s="21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G18" s="23" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="H18" s="23" t="n">
         <f aca="false">F18*G18</f>
+        <v>25</v>
+      </c>
+      <c r="I18" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=CW2400+conductive+silver+epoxy","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D19" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="I18" s="24" t="str">
-        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="9" t="n">
-        <f aca="false">SUM(H16:H18)</f>
-        <v>90.35</v>
-      </c>
-      <c r="I19" s="8"/>
-    </row>
-    <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-    </row>
-    <row r="22" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H19" s="23" t="n">
+        <f aca="false">F19*G19</f>
+        <v>10</v>
+      </c>
+      <c r="I19" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=23+gauge+stainless+steel+hypodermic+tubing","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E20" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F20" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="H20" s="23" t="n">
+        <f aca="false">F20*G20</f>
+        <v>10</v>
+      </c>
+      <c r="I20" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=micro+coax+cable+1mm","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E21" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="F21" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="H21" s="23" t="n">
+        <f aca="false">F21*G21</f>
+        <v>12</v>
+      </c>
+      <c r="I21" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=Hammond+1590B+diecast+aluminum+enclosure","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="21" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F22" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="23" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H22" s="23" t="n">
         <f aca="false">F22*G22</f>
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="I22" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.adafruit.com/product/324","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=DB9+connector+with+backshell","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
       <c r="F23" s="21" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="23" t="n">
-        <v>8.95</v>
+        <v>8</v>
       </c>
       <c r="H23" s="23" t="n">
         <f aca="false">F23*G23</f>
-        <v>8.95</v>
+        <v>8</v>
       </c>
       <c r="I23" s="24" t="str">
-        <f aca="false">HYPERLINK("https://adafruit.com/product/6121","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=5+core+shielded+cable+300V","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="F24" s="21" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G24" s="23" t="n">
-        <v>8</v>
+        <v>0.5</v>
       </c>
       <c r="H24" s="23" t="n">
         <f aca="false">F24*G24</f>
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="I24" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.thorlabs.com/thorproduct.cfm?partnumber=FAS125","Open")</f>
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=2.2nF+100V+film+capacitor","Open")</f>
         <v>Open</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>96</v>
+        <v>73</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="F25" s="21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G25" s="23" t="n">
-        <v>8.6</v>
+        <v>5</v>
       </c>
       <c r="H25" s="23" t="n">
         <f aca="false">F25*G25</f>
-        <v>25.8</v>
+        <v>5</v>
       </c>
       <c r="I25" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.thorlabs.com/thorproduct.cfm?partnumber=F25SSN1","Open")</f>
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=M3+heat+set+inserts+kit","Open")</f>
         <v>Open</v>
       </c>
     </row>
@@ -2291,14 +2499,14 @@
       <c r="F26" s="8"/>
       <c r="G26" s="8"/>
       <c r="H26" s="9" t="n">
-        <f aca="false">SUM(H22:H25)</f>
-        <v>72.75</v>
+        <f aca="false">SUM(H16:H25)</f>
+        <v>130</v>
       </c>
       <c r="I26" s="8"/>
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
@@ -2309,730 +2517,776 @@
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
     </row>
-    <row r="29" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B29" s="22" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="F29" s="21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G29" s="23" t="n">
-        <v>209.64</v>
+        <v>6.725</v>
       </c>
       <c r="H29" s="23" t="n">
         <f aca="false">F29*G29</f>
-        <v>419.28</v>
+        <v>33.625</v>
       </c>
       <c r="I29" s="24" t="str">
-        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://www.lcsc.com/product-detail/C50636.html","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="21" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="F30" s="21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G30" s="23" t="n">
-        <v>1.68</v>
+        <v>40</v>
       </c>
       <c r="H30" s="23" t="n">
         <f aca="false">F30*G30</f>
-        <v>5.04</v>
+        <v>40</v>
       </c>
       <c r="I30" s="24" t="str">
-        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://www.lcsc.com/","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="B31" s="22" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="F31" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G31" s="23" t="n">
         <v>2</v>
-      </c>
-      <c r="G31" s="23" t="n">
-        <v>18.26</v>
       </c>
       <c r="H31" s="23" t="n">
         <f aca="false">F31*G31</f>
-        <v>36.52</v>
+        <v>10</v>
       </c>
       <c r="I31" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.digikey.com/en/products/detail/analog-devices-inc/LT1469IN8-PBF/962892","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="B32" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="E32" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="F32" s="21" t="n">
+        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="9" t="n">
+        <f aca="false">SUM(H29:H31)</f>
+        <v>83.625</v>
+      </c>
+      <c r="I32" s="8"/>
+    </row>
+    <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B34" s="5"/>
+      <c r="C34" s="5"/>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+    </row>
+    <row r="35" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B35" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="D35" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="E35" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="F35" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G32" s="23" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="H32" s="23" t="n">
-        <f aca="false">F32*G32</f>
-        <v>31.5</v>
-      </c>
-      <c r="I32" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.sparkfun.com/teensy-4-1.html","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="9" t="n">
-        <f aca="false">SUM(H29:H32)</f>
-        <v>492.34</v>
-      </c>
-      <c r="I33" s="8"/>
-    </row>
-    <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-    </row>
-    <row r="36" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G35" s="23" t="n">
+        <v>14</v>
+      </c>
+      <c r="H35" s="23" t="n">
+        <f aca="false">F35*G35</f>
+        <v>14</v>
+      </c>
+      <c r="I35" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.adafruit.com/product/324","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="21" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="B36" s="22" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>81</v>
+        <v>128</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="F36" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36" s="23" t="n">
-        <v>30.17</v>
+        <v>8.95</v>
       </c>
       <c r="H36" s="23" t="n">
         <f aca="false">F36*G36</f>
-        <v>60.34</v>
+        <v>8.95</v>
       </c>
       <c r="I36" s="24" t="str">
-        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://adafruit.com/product/6121","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="21" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B37" s="22" t="s">
-        <v>108</v>
+        <v>135</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="D37" s="21" t="s">
-        <v>81</v>
+        <v>137</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>82</v>
+        <v>138</v>
       </c>
       <c r="F37" s="21" t="n">
         <v>3</v>
       </c>
       <c r="G37" s="23" t="n">
-        <v>0.8</v>
+        <v>8</v>
       </c>
       <c r="H37" s="23" t="n">
         <f aca="false">F37*G37</f>
-        <v>2.4</v>
+        <v>24</v>
       </c>
       <c r="I37" s="24" t="str">
-        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://www.thorlabs.com/thorproduct.cfm?partnumber=FAS125","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="21" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="B38" s="22" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="F38" s="21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38" s="23" t="n">
-        <v>5.73</v>
+        <v>8.6</v>
       </c>
       <c r="H38" s="23" t="n">
         <f aca="false">F38*G38</f>
-        <v>11.46</v>
+        <v>25.8</v>
       </c>
       <c r="I38" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.digikey.com/en/products/detail/ohmite/SM104031007FE/824190","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21" t="s">
-        <v>128</v>
-      </c>
-      <c r="B39" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="C39" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="D39" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="E39" s="22" t="s">
-        <v>130</v>
-      </c>
-      <c r="F39" s="21" t="n">
+        <f aca="false">HYPERLINK("https://www.thorlabs.com/thorproduct.cfm?partnumber=F25SSN1","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="9" t="n">
+        <f aca="false">SUM(H35:H38)</f>
+        <v>72.75</v>
+      </c>
+      <c r="I39" s="8"/>
+    </row>
+    <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B41" s="5"/>
+      <c r="C41" s="5"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+    </row>
+    <row r="42" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="B42" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="E42" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="F42" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="G39" s="23" t="n">
-        <v>2.09</v>
-      </c>
-      <c r="H39" s="23" t="n">
-        <f aca="false">F39*G39</f>
-        <v>4.18</v>
-      </c>
-      <c r="I39" s="24" t="str">
-        <f aca="false">HYPERLINK("https://octopart.com/part/keystone/11301","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="B40" s="22" t="s">
-        <v>132</v>
-      </c>
-      <c r="C40" s="22" t="s">
-        <v>133</v>
-      </c>
-      <c r="D40" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E40" s="22" t="s">
-        <v>135</v>
-      </c>
-      <c r="F40" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="23" t="n">
-        <v>7.99</v>
-      </c>
-      <c r="H40" s="23" t="n">
-        <f aca="false">F40*G40</f>
-        <v>7.99</v>
-      </c>
-      <c r="I40" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=Kirecoo+copper+foil+tape+2+inch","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="9" t="n">
-        <f aca="false">SUM(H36:H40)</f>
-        <v>86.37</v>
-      </c>
-      <c r="I41" s="8"/>
-    </row>
-    <row r="43" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B43" s="5"/>
-      <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="5"/>
-      <c r="F43" s="5"/>
-      <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-      <c r="I43" s="5"/>
+      <c r="G42" s="23" t="n">
+        <v>209.64</v>
+      </c>
+      <c r="H42" s="23" t="n">
+        <f aca="false">F42*G42</f>
+        <v>419.28</v>
+      </c>
+      <c r="I42" s="24" t="str">
+        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="B43" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="C43" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="E43" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="F43" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="G43" s="23" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="H43" s="23" t="n">
+        <f aca="false">F43*G43</f>
+        <v>5.04</v>
+      </c>
+      <c r="I43" s="24" t="str">
+        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
+        <v>Open</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="21" t="s">
-        <v>36</v>
+        <v>151</v>
       </c>
       <c r="B44" s="22" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D44" s="21" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="F44" s="21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G44" s="23" t="n">
-        <v>19.99</v>
+        <v>18.26</v>
       </c>
       <c r="H44" s="23" t="n">
         <f aca="false">F44*G44</f>
-        <v>19.99</v>
+        <v>36.52</v>
       </c>
       <c r="I44" s="24" t="str">
-        <f aca="false">HYPERLINK("https://store.sunlu.com/products/petg-cfpetg-carbon-fiber-3d-printer-filament-1kg","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://www.digikey.com/en/products/detail/analog-devices-inc/LT1469IN8-PBF/962892","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="21" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="B45" s="22" t="s">
-        <v>142</v>
+        <v>156</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="D45" s="21" t="s">
-        <v>134</v>
+        <v>157</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>144</v>
+        <v>158</v>
       </c>
       <c r="F45" s="21" t="n">
         <v>1</v>
       </c>
       <c r="G45" s="23" t="n">
-        <v>9.99</v>
+        <v>31.5</v>
       </c>
       <c r="H45" s="23" t="n">
         <f aca="false">F45*G45</f>
-        <v>9.99</v>
+        <v>31.5</v>
       </c>
       <c r="I45" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=uxcell+4.6mm+steel+balls+100","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="21" t="s">
-        <v>145</v>
-      </c>
-      <c r="B46" s="22" t="s">
-        <v>146</v>
-      </c>
-      <c r="C46" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="D46" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="E46" s="22" t="s">
+        <f aca="false">HYPERLINK("https://www.sparkfun.com/teensy-4-1.html","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="8"/>
+      <c r="H46" s="9" t="n">
+        <f aca="false">SUM(H42:H45)</f>
+        <v>492.34</v>
+      </c>
+      <c r="I46" s="8"/>
+    </row>
+    <row r="48" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B48" s="5"/>
+      <c r="C48" s="5"/>
+      <c r="D48" s="5"/>
+      <c r="E48" s="5"/>
+      <c r="F48" s="5"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+    </row>
+    <row r="49" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="B49" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="D49" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="E49" s="22" t="s">
+        <v>163</v>
+      </c>
+      <c r="F49" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="23" t="n">
+        <v>30.17</v>
+      </c>
+      <c r="H49" s="23" t="n">
+        <f aca="false">F49*G49</f>
+        <v>60.34</v>
+      </c>
+      <c r="I49" s="24" t="str">
+        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="B50" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="F46" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="H46" s="23" t="n">
-        <f aca="false">F46*G46</f>
-        <v>30</v>
-      </c>
-      <c r="I46" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.tedpella.com/AFM_html/AFM.aspx","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="B47" s="22" t="s">
+      <c r="C50" s="22" t="s">
         <v>150</v>
       </c>
-      <c r="C47" s="22" t="s">
-        <v>151</v>
-      </c>
-      <c r="D47" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E47" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="F47" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" s="23" t="n">
-        <v>9.49</v>
-      </c>
-      <c r="H47" s="23" t="n">
-        <f aca="false">F47*G47</f>
-        <v>9.49</v>
-      </c>
-      <c r="I47" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=TRYMAG+small+neodymium+magnets","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="21" t="s">
+      <c r="D50" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="E50" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="F50" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="G50" s="23" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H50" s="23" t="n">
+        <f aca="false">F50*G50</f>
+        <v>2.4</v>
+      </c>
+      <c r="I50" s="24" t="str">
+        <f aca="false">HYPERLINK("https://jlcpcb.com/","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21" t="s">
+        <v>165</v>
+      </c>
+      <c r="B51" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="C51" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="D51" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="B48" s="22" t="s">
-        <v>154</v>
-      </c>
-      <c r="C48" s="22" t="s">
-        <v>155</v>
-      </c>
-      <c r="D48" s="21" t="s">
-        <v>156</v>
-      </c>
-      <c r="E48" s="22" t="s">
-        <v>157</v>
-      </c>
-      <c r="F48" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="H48" s="23" t="n">
-        <f aca="false">F48*G48</f>
-        <v>35</v>
-      </c>
-      <c r="I48" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.isolateit.com/products/sorbothane-acoustic-and-vibration-isolation-square-6-x-6-pads","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="9" t="n">
-        <f aca="false">SUM(H44:H48)</f>
-        <v>104.47</v>
-      </c>
-      <c r="I49" s="8"/>
-    </row>
-    <row r="51" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5"/>
-      <c r="I51" s="5"/>
+      <c r="E51" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="F51" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="23" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="H51" s="23" t="n">
+        <f aca="false">F51*G51</f>
+        <v>11.46</v>
+      </c>
+      <c r="I51" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.digikey.com/en/products/detail/ohmite/SM104031007FE/824190","Open")</f>
+        <v>Open</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="21" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="B52" s="22" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="D52" s="21" t="s">
-        <v>87</v>
+        <v>153</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="F52" s="21" t="n">
         <v>2</v>
       </c>
       <c r="G52" s="23" t="n">
-        <v>11.5</v>
+        <v>2.09</v>
       </c>
       <c r="H52" s="23" t="n">
         <f aca="false">F52*G52</f>
-        <v>23</v>
+        <v>4.18</v>
       </c>
       <c r="I52" s="24" t="str">
-        <f aca="false">HYPERLINK("https://adafruit.com/product/4821","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="7" t="s">
+        <f aca="false">HYPERLINK("https://octopart.com/part/keystone/11301","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="B53" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="D53" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E53" s="22" t="s">
+        <v>175</v>
+      </c>
+      <c r="F53" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="23" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="H53" s="23" t="n">
+        <f aca="false">F53*G53</f>
+        <v>7.99</v>
+      </c>
+      <c r="I53" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=Kirecoo+copper+foil+tape+2+inch","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B53" s="8"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="8"/>
-      <c r="E53" s="8"/>
-      <c r="F53" s="8"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="9" t="n">
-        <f aca="false">SUM(H52:H52)</f>
-        <v>23</v>
-      </c>
-      <c r="I53" s="8"/>
-    </row>
-    <row r="55" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-    </row>
-    <row r="56" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="21" t="s">
-        <v>164</v>
-      </c>
-      <c r="B56" s="22" t="s">
-        <v>165</v>
-      </c>
-      <c r="C56" s="22" t="s">
-        <v>166</v>
-      </c>
-      <c r="D56" s="21" t="s">
-        <v>167</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="F56" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="G56" s="23" t="n">
-        <v>21.39</v>
-      </c>
-      <c r="H56" s="23" t="n">
-        <f aca="false">F56*G56</f>
-        <v>64.17</v>
-      </c>
-      <c r="I56" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.batteryjunction.com/products/energizer-ind-9v-en22-12pk","Open")</f>
-        <v>Open</v>
-      </c>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="9" t="n">
+        <f aca="false">SUM(H49:H53)</f>
+        <v>86.37</v>
+      </c>
+      <c r="I54" s="8"/>
+    </row>
+    <row r="56" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
     </row>
     <row r="57" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="21" t="s">
-        <v>169</v>
+        <v>36</v>
       </c>
       <c r="B57" s="22" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="D57" s="21" t="s">
-        <v>112</v>
+        <v>179</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="F57" s="21" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="G57" s="23" t="n">
-        <v>0.61</v>
+        <v>19.99</v>
       </c>
       <c r="H57" s="23" t="n">
         <f aca="false">F57*G57</f>
-        <v>12.2</v>
+        <v>19.99</v>
       </c>
       <c r="I57" s="24" t="str">
-        <f aca="false">HYPERLINK("https://octopart.com/part/keystone/232","Open")</f>
+        <f aca="false">HYPERLINK("https://store.sunlu.com/products/petg-cfpetg-carbon-fiber-3d-printer-filament-1kg","Open")</f>
         <v>Open</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="21" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B58" s="22" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D58" s="21" t="s">
-        <v>167</v>
+        <v>73</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="F58" s="21" t="n">
         <v>1</v>
       </c>
       <c r="G58" s="23" t="n">
-        <v>10.95</v>
+        <v>9.99</v>
       </c>
       <c r="H58" s="23" t="n">
         <f aca="false">F58*G58</f>
-        <v>10.95</v>
+        <v>9.99</v>
       </c>
       <c r="I58" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.batteryjunction.com/products/energizer-ind-aa-en91-24pk","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=uxcell+4.6mm+steel+balls+100","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="21" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B59" s="22" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D59" s="21" t="s">
-        <v>87</v>
+        <v>188</v>
       </c>
       <c r="E59" s="22" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="F59" s="21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G59" s="23" t="n">
-        <v>2.95</v>
+        <v>30</v>
       </c>
       <c r="H59" s="23" t="n">
         <f aca="false">F59*G59</f>
-        <v>5.9</v>
+        <v>30</v>
       </c>
       <c r="I59" s="24" t="str">
-        <f aca="false">HYPERLINK("https://www.adafruit.com/product/449","Open")</f>
-        <v>Open</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B60" s="8"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="8"/>
-      <c r="E60" s="8"/>
-      <c r="F60" s="8"/>
-      <c r="G60" s="8"/>
-      <c r="H60" s="9" t="n">
-        <f aca="false">SUM(H56:H59)</f>
-        <v>93.22</v>
-      </c>
-      <c r="I60" s="8"/>
+        <f aca="false">HYPERLINK("https://www.tedpella.com/AFM_html/AFM.aspx","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B60" s="22" t="s">
+        <v>190</v>
+      </c>
+      <c r="C60" s="22" t="s">
+        <v>191</v>
+      </c>
+      <c r="D60" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E60" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="F60" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="23" t="n">
+        <v>9.49</v>
+      </c>
+      <c r="H60" s="23" t="n">
+        <f aca="false">F60*G60</f>
+        <v>9.49</v>
+      </c>
+      <c r="I60" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=TRYMAG+small+neodymium+magnets","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="B61" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="C61" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="D61" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="E61" s="22" t="s">
+        <v>197</v>
+      </c>
+      <c r="F61" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="H61" s="23" t="n">
+        <f aca="false">F61*G61</f>
+        <v>35</v>
+      </c>
+      <c r="I61" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.isolateit.com/products/sorbothane-acoustic-and-vibration-isolation-square-6-x-6-pads","Open")</f>
+        <v>Open</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>181</v>
+        <v>15</v>
       </c>
       <c r="B62" s="8"/>
       <c r="C62" s="8"/>
@@ -3041,47 +3295,58 @@
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
       <c r="H62" s="9" t="n">
-        <f aca="false">H13+H19+H26+H33+H41+H49+H53+H60</f>
-        <v>1093.5</v>
+        <f aca="false">SUM(H57:H61)</f>
+        <v>104.47</v>
       </c>
       <c r="I62" s="8"/>
     </row>
-    <row r="63" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B63" s="22" t="s">
-        <v>182</v>
-      </c>
-      <c r="H63" s="6" t="n">
-        <v>166.75</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="0" t="s">
-        <v>183</v>
-      </c>
-      <c r="B64" s="22" t="s">
-        <v>184</v>
-      </c>
-      <c r="H64" s="6" t="n">
-        <v>202.09</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="0" t="s">
-        <v>185</v>
+    <row r="64" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="B64" s="5"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+      <c r="I64" s="5"/>
+    </row>
+    <row r="65" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="21" t="s">
+        <v>199</v>
       </c>
       <c r="B65" s="22" t="s">
-        <v>186</v>
-      </c>
-      <c r="H65" s="6" t="n">
-        <v>83.25</v>
+        <v>200</v>
+      </c>
+      <c r="C65" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="D65" s="21" t="s">
+        <v>128</v>
+      </c>
+      <c r="E65" s="22" t="s">
+        <v>202</v>
+      </c>
+      <c r="F65" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G65" s="23" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="H65" s="23" t="n">
+        <f aca="false">F65*G65</f>
+        <v>23</v>
+      </c>
+      <c r="I65" s="24" t="str">
+        <f aca="false">HYPERLINK("https://adafruit.com/product/4821","Open")</f>
+        <v>Open</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>187</v>
+        <v>15</v>
       </c>
       <c r="B66" s="8"/>
       <c r="C66" s="8"/>
@@ -3090,636 +3355,918 @@
       <c r="F66" s="8"/>
       <c r="G66" s="8"/>
       <c r="H66" s="9" t="n">
-        <f aca="false">SUM(H63:H65)</f>
-        <v>452.09</v>
+        <f aca="false">SUM(H65:H65)</f>
+        <v>23</v>
       </c>
       <c r="I66" s="8"/>
     </row>
-    <row r="67" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="25" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="26" t="s">
-        <v>189</v>
-      </c>
-      <c r="B69" s="27"/>
-      <c r="C69" s="27"/>
-      <c r="D69" s="27"/>
-      <c r="E69" s="27"/>
-      <c r="F69" s="27"/>
-      <c r="G69" s="27"/>
-      <c r="H69" s="27"/>
-      <c r="I69" s="27"/>
-      <c r="J69" s="27"/>
-    </row>
-    <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="28" t="s">
-        <v>2</v>
-      </c>
-      <c r="B70" s="28" t="s">
-        <v>56</v>
-      </c>
-      <c r="C70" s="28" t="s">
-        <v>57</v>
-      </c>
-      <c r="D70" s="28" t="s">
-        <v>58</v>
-      </c>
-      <c r="E70" s="28" t="s">
-        <v>59</v>
-      </c>
-      <c r="F70" s="28" t="s">
+    <row r="68" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5"/>
+      <c r="I68" s="5"/>
+    </row>
+    <row r="69" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="B69" s="22" t="s">
+        <v>205</v>
+      </c>
+      <c r="C69" s="22" t="s">
+        <v>206</v>
+      </c>
+      <c r="D69" s="21" t="s">
+        <v>207</v>
+      </c>
+      <c r="E69" s="22" t="s">
+        <v>208</v>
+      </c>
+      <c r="F69" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="G70" s="28" t="s">
-        <v>60</v>
-      </c>
-      <c r="H70" s="28" t="s">
-        <v>61</v>
-      </c>
-      <c r="I70" s="28" t="s">
-        <v>62</v>
-      </c>
-      <c r="J70" s="28" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G69" s="23" t="n">
+        <v>21.39</v>
+      </c>
+      <c r="H69" s="23" t="n">
+        <f aca="false">F69*G69</f>
+        <v>64.17</v>
+      </c>
+      <c r="I69" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.batteryjunction.com/products/energizer-ind-9v-en22-12pk","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="B70" s="22" t="s">
+        <v>210</v>
+      </c>
+      <c r="C70" s="22" t="s">
+        <v>211</v>
+      </c>
+      <c r="D70" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="E70" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="F70" s="21" t="n">
+        <v>20</v>
+      </c>
+      <c r="G70" s="23" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="H70" s="23" t="n">
+        <f aca="false">F70*G70</f>
+        <v>12.2</v>
+      </c>
+      <c r="I70" s="24" t="str">
+        <f aca="false">HYPERLINK("https://octopart.com/part/keystone/232","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="21" t="s">
-        <v>191</v>
+        <v>213</v>
       </c>
       <c r="B71" s="22" t="s">
-        <v>192</v>
+        <v>214</v>
       </c>
       <c r="C71" s="22" t="s">
-        <v>193</v>
+        <v>215</v>
       </c>
       <c r="D71" s="21" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="E71" s="22" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="F71" s="21" t="n">
         <v>1</v>
       </c>
       <c r="G71" s="23" t="n">
-        <v>277.2</v>
+        <v>10.95</v>
       </c>
       <c r="H71" s="23" t="n">
-        <f aca="false">IF(OR(J71="Yes",J71=TRUE()),0,F71*G71)</f>
-        <v>277.2</v>
+        <f aca="false">F71*G71</f>
+        <v>10.95</v>
       </c>
       <c r="I71" s="24" t="str">
-        <f aca="false">HYPERLINK("https://store.bruker.com/products/dpt10","Open")</f>
-        <v>Open</v>
-      </c>
-      <c r="J71" s="29"/>
+        <f aca="false">HYPERLINK("https://www.batteryjunction.com/products/energizer-ind-aa-en91-24pk","Open")</f>
+        <v>Open</v>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="21" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="B72" s="22" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="C72" s="22" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="D72" s="21" t="s">
-        <v>199</v>
+        <v>128</v>
       </c>
       <c r="E72" s="22" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="F72" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G72" s="23" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="H72" s="23" t="n">
+        <f aca="false">F72*G72</f>
+        <v>5.9</v>
+      </c>
+      <c r="I72" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.adafruit.com/product/449","Open")</f>
+        <v>Open</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B73" s="8"/>
+      <c r="C73" s="8"/>
+      <c r="D73" s="8"/>
+      <c r="E73" s="8"/>
+      <c r="F73" s="8"/>
+      <c r="G73" s="8"/>
+      <c r="H73" s="9" t="n">
+        <f aca="false">SUM(H69:H72)</f>
+        <v>93.22</v>
+      </c>
+      <c r="I73" s="8"/>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="B75" s="8"/>
+      <c r="C75" s="8"/>
+      <c r="D75" s="8"/>
+      <c r="E75" s="8"/>
+      <c r="F75" s="8"/>
+      <c r="G75" s="8"/>
+      <c r="H75" s="9" t="n">
+        <f aca="false">H13+H26+H32+H39+H46+H54+H62+H66+H73</f>
+        <v>1216.775</v>
+      </c>
+      <c r="I75" s="8"/>
+    </row>
+    <row r="76" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B76" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="H76" s="6" t="n">
+        <v>166.75</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="0" t="s">
+        <v>223</v>
+      </c>
+      <c r="B77" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="H77" s="6" t="n">
+        <v>199.74</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="0" t="s">
+        <v>225</v>
+      </c>
+      <c r="B78" s="22" t="s">
+        <v>226</v>
+      </c>
+      <c r="H78" s="6" t="n">
+        <v>83.25</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="B79" s="8"/>
+      <c r="C79" s="8"/>
+      <c r="D79" s="8"/>
+      <c r="E79" s="8"/>
+      <c r="F79" s="8"/>
+      <c r="G79" s="8"/>
+      <c r="H79" s="9" t="n">
+        <f aca="false">SUM(H76:H78)</f>
+        <v>449.74</v>
+      </c>
+      <c r="I79" s="8"/>
+    </row>
+    <row r="80" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B80" s="25" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="26" t="s">
+        <v>229</v>
+      </c>
+      <c r="B82" s="27"/>
+      <c r="C82" s="27"/>
+      <c r="D82" s="27"/>
+      <c r="E82" s="27"/>
+      <c r="F82" s="27"/>
+      <c r="G82" s="27"/>
+      <c r="H82" s="27"/>
+      <c r="I82" s="27"/>
+      <c r="J82" s="27"/>
+    </row>
+    <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A83" s="28" t="s">
+        <v>2</v>
+      </c>
+      <c r="B83" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="C83" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="D83" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="E83" s="28" t="s">
+        <v>59</v>
+      </c>
+      <c r="F83" s="28" t="s">
+        <v>3</v>
+      </c>
+      <c r="G83" s="28" t="s">
+        <v>60</v>
+      </c>
+      <c r="H83" s="28" t="s">
+        <v>61</v>
+      </c>
+      <c r="I83" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="J83" s="28" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="21" t="s">
+        <v>231</v>
+      </c>
+      <c r="B84" s="22" t="s">
+        <v>232</v>
+      </c>
+      <c r="C84" s="22" t="s">
+        <v>233</v>
+      </c>
+      <c r="D84" s="21" t="s">
+        <v>234</v>
+      </c>
+      <c r="E84" s="22" t="s">
+        <v>235</v>
+      </c>
+      <c r="F84" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G72" s="23" t="n">
+      <c r="G84" s="23" t="n">
+        <v>277.2</v>
+      </c>
+      <c r="H84" s="23" t="n">
+        <f aca="false">IF(OR(J84="Yes",J84=TRUE()),0,F84*G84)</f>
+        <v>277.2</v>
+      </c>
+      <c r="I84" s="24" t="str">
+        <f aca="false">HYPERLINK("https://store.bruker.com/products/dpt10","Open")</f>
+        <v>Open</v>
+      </c>
+      <c r="J84" s="29"/>
+    </row>
+    <row r="85" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="B85" s="22" t="s">
+        <v>237</v>
+      </c>
+      <c r="C85" s="22" t="s">
+        <v>238</v>
+      </c>
+      <c r="D85" s="21" t="s">
+        <v>239</v>
+      </c>
+      <c r="E85" s="22" t="s">
+        <v>240</v>
+      </c>
+      <c r="F85" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="23" t="n">
         <v>77</v>
       </c>
-      <c r="H72" s="23" t="n">
-        <f aca="false">IF(OR(J72="Yes",J72=TRUE()),0,F72*G72)</f>
+      <c r="H85" s="23" t="n">
+        <f aca="false">IF(OR(J85="Yes",J85=TRUE()),0,F85*G85)</f>
         <v>77</v>
       </c>
-      <c r="I72" s="24" t="str">
+      <c r="I85" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.nanoandmore.com/AFM-Accessories-HOPG-ZYH","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J72" s="29"/>
-    </row>
-    <row r="73" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="21" t="s">
-        <v>201</v>
-      </c>
-      <c r="B73" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="C73" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="D73" s="21" t="s">
-        <v>204</v>
-      </c>
-      <c r="E73" s="22" t="s">
-        <v>205</v>
-      </c>
-      <c r="F73" s="21" t="n">
+      <c r="J85" s="29"/>
+    </row>
+    <row r="86" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="B86" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="C86" s="22" t="s">
+        <v>243</v>
+      </c>
+      <c r="D86" s="21" t="s">
+        <v>244</v>
+      </c>
+      <c r="E86" s="22" t="s">
+        <v>245</v>
+      </c>
+      <c r="F86" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G73" s="23" t="n">
+      <c r="G86" s="23" t="n">
         <v>133.13</v>
       </c>
-      <c r="H73" s="23" t="n">
-        <f aca="false">IF(OR(J73="Yes",J73=TRUE()),0,F73*G73)</f>
+      <c r="H86" s="23" t="n">
+        <f aca="false">IF(OR(J86="Yes",J86=TRUE()),0,F86*G86)</f>
         <v>133.13</v>
       </c>
-      <c r="I73" s="24" t="str">
+      <c r="I86" s="24" t="str">
         <f aca="false">HYPERLINK("https://octopart.com/search?q=8331D-14G","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J73" s="29"/>
-    </row>
-    <row r="74" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="B74" s="22" t="s">
-        <v>207</v>
-      </c>
-      <c r="C74" s="22" t="s">
-        <v>208</v>
-      </c>
-      <c r="D74" s="21" t="s">
-        <v>209</v>
-      </c>
-      <c r="E74" s="22" t="s">
-        <v>210</v>
-      </c>
-      <c r="F74" s="21" t="n">
+      <c r="J86" s="29"/>
+    </row>
+    <row r="87" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="21" t="s">
+        <v>246</v>
+      </c>
+      <c r="B87" s="22" t="s">
+        <v>247</v>
+      </c>
+      <c r="C87" s="22" t="s">
+        <v>248</v>
+      </c>
+      <c r="D87" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="E87" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="F87" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G74" s="23" t="n">
+      <c r="G87" s="23" t="n">
         <v>75.15</v>
       </c>
-      <c r="H74" s="23" t="n">
-        <f aca="false">IF(OR(J74="Yes",J74=TRUE()),0,F74*G74)</f>
+      <c r="H87" s="23" t="n">
+        <f aca="false">IF(OR(J87="Yes",J87=TRUE()),0,F87*G87)</f>
         <v>75.15</v>
       </c>
-      <c r="I74" s="24" t="str">
+      <c r="I87" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.penntoolco.com/grizzly-9-x-12-x-2-granite-surface-plate-no-ledge-g9649/","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J74" s="29"/>
-    </row>
-    <row r="75" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="21" t="s">
+      <c r="J87" s="29"/>
+    </row>
+    <row r="88" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="B75" s="22" t="s">
-        <v>211</v>
-      </c>
-      <c r="C75" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D75" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E75" s="22" t="s">
-        <v>213</v>
-      </c>
-      <c r="F75" s="21" t="n">
+      <c r="B88" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="C88" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D88" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E88" s="22" t="s">
+        <v>253</v>
+      </c>
+      <c r="F88" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G75" s="23" t="n">
+      <c r="G88" s="23" t="n">
         <v>57.99</v>
       </c>
-      <c r="H75" s="23" t="n">
-        <f aca="false">IF(OR(J75="Yes",J75=TRUE()),0,F75*G75)</f>
+      <c r="H88" s="23" t="n">
+        <f aca="false">IF(OR(J88="Yes",J88=TRUE()),0,F88*G88)</f>
         <v>57.99</v>
       </c>
-      <c r="I75" s="24" t="str">
+      <c r="I88" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=FNIRSI+DST-201+oscilloscope+multimeter","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J75" s="29"/>
-    </row>
-    <row r="76" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="21" t="s">
-        <v>214</v>
-      </c>
-      <c r="B76" s="22" t="s">
-        <v>215</v>
-      </c>
-      <c r="C76" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D76" s="21" t="s">
-        <v>216</v>
-      </c>
-      <c r="E76" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="F76" s="21" t="n">
+      <c r="J88" s="29"/>
+    </row>
+    <row r="89" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="21" t="s">
+        <v>254</v>
+      </c>
+      <c r="B89" s="22" t="s">
+        <v>255</v>
+      </c>
+      <c r="C89" s="22" t="s">
+        <v>256</v>
+      </c>
+      <c r="D89" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E89" s="22" t="s">
+        <v>257</v>
+      </c>
+      <c r="F89" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G76" s="23" t="n">
+      <c r="G89" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="H89" s="23" t="n">
+        <f aca="false">IF(OR(J89="Yes",J89=TRUE()),0,F89*G89)</f>
+        <v>40</v>
+      </c>
+      <c r="I89" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=handheld+LCR+meter","Open")</f>
+        <v>Open</v>
+      </c>
+      <c r="J89" s="29"/>
+    </row>
+    <row r="90" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="21" t="s">
+        <v>258</v>
+      </c>
+      <c r="B90" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="C90" s="22" t="s">
+        <v>260</v>
+      </c>
+      <c r="D90" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E90" s="22" t="s">
+        <v>261</v>
+      </c>
+      <c r="F90" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G90" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="H90" s="23" t="n">
+        <f aca="false">IF(OR(J90="Yes",J90=TRUE()),0,F90*G90)</f>
+        <v>60</v>
+      </c>
+      <c r="I90" s="24" t="str">
+        <f aca="false">HYPERLINK("https://www.amazon.com/s?k=Michelson+interferometer+kit+beamsplitter+cube+laser+diode","Open")</f>
+        <v>Open</v>
+      </c>
+      <c r="J90" s="29"/>
+    </row>
+    <row r="91" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="21" t="s">
+        <v>262</v>
+      </c>
+      <c r="B91" s="22" t="s">
+        <v>263</v>
+      </c>
+      <c r="C91" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D91" s="21" t="s">
+        <v>264</v>
+      </c>
+      <c r="E91" s="22" t="s">
+        <v>265</v>
+      </c>
+      <c r="F91" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G91" s="23" t="n">
         <v>25.99</v>
       </c>
-      <c r="H76" s="23" t="n">
-        <f aca="false">IF(OR(J76="Yes",J76=TRUE()),0,F76*G76)</f>
+      <c r="H91" s="23" t="n">
+        <f aca="false">IF(OR(J91="Yes",J91=TRUE()),0,F91*G91)</f>
         <v>25.99</v>
       </c>
-      <c r="I76" s="24" t="str">
+      <c r="I91" s="24" t="str">
         <f aca="false">HYPERLINK("https://pine64.com/?p=158078","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J76" s="29"/>
-    </row>
-    <row r="77" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="21" t="s">
-        <v>218</v>
-      </c>
-      <c r="B77" s="22" t="s">
-        <v>219</v>
-      </c>
-      <c r="C77" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D77" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E77" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F77" s="21" t="n">
+      <c r="J91" s="29"/>
+    </row>
+    <row r="92" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="21" t="s">
+        <v>266</v>
+      </c>
+      <c r="B92" s="22" t="s">
+        <v>267</v>
+      </c>
+      <c r="C92" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D92" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E92" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="F92" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G77" s="23" t="n">
+      <c r="G92" s="23" t="n">
         <v>24.97</v>
       </c>
-      <c r="H77" s="23" t="n">
-        <f aca="false">IF(OR(J77="Yes",J77=TRUE()),0,F77*G77)</f>
+      <c r="H92" s="23" t="n">
+        <f aca="false">IF(OR(J92="Yes",J92=TRUE()),0,F92*G92)</f>
         <v>24.97</v>
       </c>
-      <c r="I77" s="24" t="str">
+      <c r="I92" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=Sn42Bi58+solder+paste","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J77" s="29"/>
-    </row>
-    <row r="78" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="21" t="s">
-        <v>221</v>
-      </c>
-      <c r="B78" s="22" t="s">
-        <v>222</v>
-      </c>
-      <c r="C78" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D78" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E78" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F78" s="21" t="n">
+      <c r="J92" s="29"/>
+    </row>
+    <row r="93" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="21" t="s">
+        <v>269</v>
+      </c>
+      <c r="B93" s="22" t="s">
+        <v>270</v>
+      </c>
+      <c r="C93" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D93" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E93" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="F93" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G78" s="23" t="n">
+      <c r="G93" s="23" t="n">
         <v>11.99</v>
       </c>
-      <c r="H78" s="23" t="n">
-        <f aca="false">IF(OR(J78="Yes",J78=TRUE()),0,F78*G78)</f>
+      <c r="H93" s="23" t="n">
+        <f aca="false">IF(OR(J93="Yes",J93=TRUE()),0,F93*G93)</f>
         <v>11.99</v>
       </c>
-      <c r="I78" s="24" t="str">
+      <c r="I93" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=heat+shrink+tubing+kit","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J78" s="29"/>
-    </row>
-    <row r="79" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="B79" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="C79" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D79" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E79" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F79" s="21" t="n">
+      <c r="J93" s="29"/>
+    </row>
+    <row r="94" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="21" t="s">
+        <v>271</v>
+      </c>
+      <c r="B94" s="22" t="s">
+        <v>272</v>
+      </c>
+      <c r="C94" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D94" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E94" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="F94" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G79" s="23" t="n">
+      <c r="G94" s="23" t="n">
         <v>25.26</v>
       </c>
-      <c r="H79" s="23" t="n">
-        <f aca="false">IF(OR(J79="Yes",J79=TRUE()),0,F79*G79)</f>
+      <c r="H94" s="23" t="n">
+        <f aca="false">IF(OR(J94="Yes",J94=TRUE()),0,F94*G94)</f>
         <v>25.26</v>
       </c>
-      <c r="I79" s="24" t="str">
+      <c r="I94" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=RG178+coax+cable","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J79" s="29"/>
-    </row>
-    <row r="80" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="21" t="s">
-        <v>225</v>
-      </c>
-      <c r="B80" s="22" t="s">
-        <v>226</v>
-      </c>
-      <c r="C80" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D80" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E80" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F80" s="21" t="n">
+      <c r="J94" s="29"/>
+    </row>
+    <row r="95" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="21" t="s">
+        <v>273</v>
+      </c>
+      <c r="B95" s="22" t="s">
+        <v>274</v>
+      </c>
+      <c r="C95" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D95" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E95" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="F95" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G80" s="23" t="n">
+      <c r="G95" s="23" t="n">
         <v>32.12</v>
       </c>
-      <c r="H80" s="23" t="n">
-        <f aca="false">IF(OR(J80="Yes",J80=TRUE()),0,F80*G80)</f>
+      <c r="H95" s="23" t="n">
+        <f aca="false">IF(OR(J95="Yes",J95=TRUE()),0,F95*G95)</f>
         <v>32.12</v>
       </c>
-      <c r="I80" s="24" t="str">
+      <c r="I95" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=2x13+IDC+ribbon+cable","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J80" s="29"/>
-    </row>
-    <row r="81" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="21" t="s">
-        <v>227</v>
-      </c>
-      <c r="B81" s="22" t="s">
-        <v>228</v>
-      </c>
-      <c r="C81" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D81" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E81" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F81" s="21" t="n">
+      <c r="J95" s="29"/>
+    </row>
+    <row r="96" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="21" t="s">
+        <v>275</v>
+      </c>
+      <c r="B96" s="22" t="s">
+        <v>276</v>
+      </c>
+      <c r="C96" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D96" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E96" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="F96" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G81" s="23" t="n">
+      <c r="G96" s="23" t="n">
         <v>16.98</v>
       </c>
-      <c r="H81" s="23" t="n">
-        <f aca="false">IF(OR(J81="Yes",J81=TRUE()),0,F81*G81)</f>
+      <c r="H96" s="23" t="n">
+        <f aca="false">IF(OR(J96="Yes",J96=TRUE()),0,F96*G96)</f>
         <v>16.98</v>
       </c>
-      <c r="I81" s="24" t="str">
+      <c r="I96" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=pin+header+kit","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J81" s="29"/>
-    </row>
-    <row r="82" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="21" t="s">
-        <v>229</v>
-      </c>
-      <c r="B82" s="22" t="s">
-        <v>230</v>
-      </c>
-      <c r="C82" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D82" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E82" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F82" s="21" t="n">
+      <c r="J96" s="29"/>
+    </row>
+    <row r="97" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="21" t="s">
+        <v>277</v>
+      </c>
+      <c r="B97" s="22" t="s">
+        <v>278</v>
+      </c>
+      <c r="C97" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D97" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E97" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="F97" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G82" s="23" t="n">
+      <c r="G97" s="23" t="n">
         <v>22.31</v>
       </c>
-      <c r="H82" s="23" t="n">
-        <f aca="false">IF(OR(J82="Yes",J82=TRUE()),0,F82*G82)</f>
+      <c r="H97" s="23" t="n">
+        <f aca="false">IF(OR(J97="Yes",J97=TRUE()),0,F97*G97)</f>
         <v>22.31</v>
       </c>
-      <c r="I82" s="24" t="str">
+      <c r="I97" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=M2+M2.5+M3+screw+kit","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J82" s="29"/>
-    </row>
-    <row r="83" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="21" t="s">
-        <v>231</v>
-      </c>
-      <c r="B83" s="22" t="s">
-        <v>232</v>
-      </c>
-      <c r="C83" s="22" t="s">
-        <v>212</v>
-      </c>
-      <c r="D83" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="E83" s="22" t="s">
-        <v>220</v>
-      </c>
-      <c r="F83" s="21" t="n">
+      <c r="J97" s="29"/>
+    </row>
+    <row r="98" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="21" t="s">
+        <v>279</v>
+      </c>
+      <c r="B98" s="22" t="s">
+        <v>280</v>
+      </c>
+      <c r="C98" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="D98" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E98" s="22" t="s">
+        <v>268</v>
+      </c>
+      <c r="F98" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="G83" s="23" t="n">
+      <c r="G98" s="23" t="n">
         <v>12.17</v>
       </c>
-      <c r="H83" s="23" t="n">
-        <f aca="false">IF(OR(J83="Yes",J83=TRUE()),0,F83*G83)</f>
+      <c r="H98" s="23" t="n">
+        <f aca="false">IF(OR(J98="Yes",J98=TRUE()),0,F98*G98)</f>
         <v>12.17</v>
       </c>
-      <c r="I83" s="24" t="str">
+      <c r="I98" s="24" t="str">
         <f aca="false">HYPERLINK("https://www.amazon.com/s?k=precision+tweezers+set","Open")</f>
         <v>Open</v>
       </c>
-      <c r="J83" s="29"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="30" t="s">
-        <v>233</v>
-      </c>
-      <c r="B84" s="31"/>
-      <c r="C84" s="31"/>
-      <c r="D84" s="31"/>
-      <c r="E84" s="31"/>
-      <c r="F84" s="31"/>
-      <c r="G84" s="31"/>
-      <c r="H84" s="32" t="n">
-        <f aca="false">SUM(H71:H83)</f>
-        <v>792.26</v>
-      </c>
-      <c r="I84" s="31"/>
-      <c r="J84" s="31"/>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="B86" s="33"/>
-      <c r="C86" s="33"/>
-      <c r="D86" s="33"/>
-      <c r="E86" s="33"/>
-      <c r="F86" s="33"/>
-      <c r="G86" s="33"/>
-      <c r="H86" s="33"/>
-      <c r="I86" s="33"/>
-      <c r="J86" s="33"/>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="34" t="s">
-        <v>235</v>
-      </c>
-      <c r="B87" s="35" t="s">
-        <v>236</v>
-      </c>
-      <c r="C87" s="36"/>
-      <c r="D87" s="36"/>
-      <c r="E87" s="36"/>
-      <c r="F87" s="36"/>
-      <c r="G87" s="36"/>
-      <c r="H87" s="37" t="n">
-        <f aca="false">H62+H84</f>
-        <v>1885.76</v>
-      </c>
-      <c r="I87" s="36"/>
-      <c r="J87" s="36"/>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="34" t="s">
-        <v>237</v>
-      </c>
-      <c r="B88" s="35"/>
-      <c r="C88" s="36"/>
-      <c r="D88" s="36"/>
-      <c r="E88" s="36"/>
-      <c r="F88" s="36"/>
-      <c r="G88" s="36"/>
-      <c r="H88" s="37" t="n">
-        <f aca="false">H66</f>
-        <v>452.09</v>
-      </c>
-      <c r="I88" s="36"/>
-      <c r="J88" s="36"/>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="34" t="s">
-        <v>238</v>
-      </c>
-      <c r="B89" s="35"/>
-      <c r="C89" s="36"/>
-      <c r="D89" s="36"/>
-      <c r="E89" s="36"/>
-      <c r="F89" s="36"/>
-      <c r="G89" s="36"/>
-      <c r="H89" s="37" t="n">
-        <f aca="false">ROUND(H87*0.0775,2)</f>
-        <v>146.15</v>
-      </c>
-      <c r="I89" s="36"/>
-      <c r="J89" s="36"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="34" t="s">
-        <v>239</v>
-      </c>
-      <c r="B90" s="35"/>
-      <c r="C90" s="36"/>
-      <c r="D90" s="36"/>
-      <c r="E90" s="36"/>
-      <c r="F90" s="36"/>
-      <c r="G90" s="36"/>
-      <c r="H90" s="37" t="n">
-        <f aca="false">ROUND((H87+H88+H89)*0.1,2)</f>
-        <v>248.4</v>
-      </c>
-      <c r="I90" s="36"/>
-      <c r="J90" s="36"/>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="B91" s="38"/>
-      <c r="C91" s="12"/>
-      <c r="D91" s="12"/>
-      <c r="E91" s="12"/>
-      <c r="F91" s="12"/>
-      <c r="G91" s="12"/>
-      <c r="H91" s="13" t="n">
-        <f aca="false">H87+H88+H89+H90</f>
-        <v>2732.4</v>
-      </c>
-      <c r="I91" s="12"/>
-      <c r="J91" s="12"/>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="34" t="s">
-        <v>241</v>
-      </c>
-      <c r="B92" s="35" t="s">
-        <v>242</v>
-      </c>
-      <c r="C92" s="36"/>
-      <c r="D92" s="36"/>
-      <c r="E92" s="36"/>
-      <c r="F92" s="36"/>
-      <c r="G92" s="36"/>
-      <c r="H92" s="37" t="n">
-        <f aca="false">2000-H91</f>
-        <v>-732.4</v>
-      </c>
-      <c r="I92" s="36"/>
-      <c r="J92" s="36"/>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="2" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="H95" s="39" t="n">
-        <f aca="false">ROUND((H62+ROUND(H62*0.0775,2)+H66)*1.1,2)</f>
-        <v>1793.37</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="H96" s="39" t="n">
-        <f aca="false">ROUND((H62+SUMPRODUCT(F71:F83,G71:G83))*1.0775*1.1+H66*1.1,2)</f>
-        <v>2732.4</v>
+      <c r="J98" s="29"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="30" t="s">
+        <v>281</v>
+      </c>
+      <c r="B99" s="31"/>
+      <c r="C99" s="31"/>
+      <c r="D99" s="31"/>
+      <c r="E99" s="31"/>
+      <c r="F99" s="31"/>
+      <c r="G99" s="31"/>
+      <c r="H99" s="32" t="n">
+        <f aca="false">SUM(H84:H98)</f>
+        <v>892.26</v>
+      </c>
+      <c r="I99" s="31"/>
+      <c r="J99" s="31"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B101" s="33"/>
+      <c r="C101" s="33"/>
+      <c r="D101" s="33"/>
+      <c r="E101" s="33"/>
+      <c r="F101" s="33"/>
+      <c r="G101" s="33"/>
+      <c r="H101" s="33"/>
+      <c r="I101" s="33"/>
+      <c r="J101" s="33"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="34" t="s">
+        <v>283</v>
+      </c>
+      <c r="B102" s="35" t="s">
+        <v>284</v>
+      </c>
+      <c r="C102" s="36"/>
+      <c r="D102" s="36"/>
+      <c r="E102" s="36"/>
+      <c r="F102" s="36"/>
+      <c r="G102" s="36"/>
+      <c r="H102" s="37" t="n">
+        <f aca="false">H75+H99</f>
+        <v>2109.035</v>
+      </c>
+      <c r="I102" s="36"/>
+      <c r="J102" s="36"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="34" t="s">
+        <v>285</v>
+      </c>
+      <c r="B103" s="35"/>
+      <c r="C103" s="36"/>
+      <c r="D103" s="36"/>
+      <c r="E103" s="36"/>
+      <c r="F103" s="36"/>
+      <c r="G103" s="36"/>
+      <c r="H103" s="37" t="n">
+        <f aca="false">H79</f>
+        <v>449.74</v>
+      </c>
+      <c r="I103" s="36"/>
+      <c r="J103" s="36"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="34" t="s">
+        <v>286</v>
+      </c>
+      <c r="B104" s="35"/>
+      <c r="C104" s="36"/>
+      <c r="D104" s="36"/>
+      <c r="E104" s="36"/>
+      <c r="F104" s="36"/>
+      <c r="G104" s="36"/>
+      <c r="H104" s="37" t="n">
+        <f aca="false">ROUND(H102*0.0775,2)</f>
+        <v>163.45</v>
+      </c>
+      <c r="I104" s="36"/>
+      <c r="J104" s="36"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="34" t="s">
+        <v>287</v>
+      </c>
+      <c r="B105" s="35"/>
+      <c r="C105" s="36"/>
+      <c r="D105" s="36"/>
+      <c r="E105" s="36"/>
+      <c r="F105" s="36"/>
+      <c r="G105" s="36"/>
+      <c r="H105" s="37" t="n">
+        <f aca="false">ROUND((H102+H103+H104)*0.1,2)</f>
+        <v>272.22</v>
+      </c>
+      <c r="I105" s="36"/>
+      <c r="J105" s="36"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="11" t="s">
+        <v>288</v>
+      </c>
+      <c r="B106" s="38"/>
+      <c r="C106" s="12"/>
+      <c r="D106" s="12"/>
+      <c r="E106" s="12"/>
+      <c r="F106" s="12"/>
+      <c r="G106" s="12"/>
+      <c r="H106" s="13" t="n">
+        <f aca="false">H102+H103+H104+H105</f>
+        <v>2994.445</v>
+      </c>
+      <c r="I106" s="12"/>
+      <c r="J106" s="12"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="34" t="s">
+        <v>289</v>
+      </c>
+      <c r="B107" s="35" t="s">
+        <v>290</v>
+      </c>
+      <c r="C107" s="36"/>
+      <c r="D107" s="36"/>
+      <c r="E107" s="36"/>
+      <c r="F107" s="36"/>
+      <c r="G107" s="36"/>
+      <c r="H107" s="37" t="n">
+        <f aca="false">2000-H106</f>
+        <v>-994.445</v>
+      </c>
+      <c r="I107" s="36"/>
+      <c r="J107" s="36"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="H110" s="39" t="n">
+        <f aca="false">ROUND((H75+ROUND(H75*0.0775,2)+H79)*1.1,2)</f>
+        <v>1936.9</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="H111" s="39" t="n">
+        <f aca="false">ROUND((H75+SUMPRODUCT(F84:F98,G84:G98))*1.0775*1.1+H79*1.1,2)</f>
+        <v>2994.45</v>
       </c>
     </row>
   </sheetData>
@@ -3731,7 +4278,7 @@
     <mergeCell ref="A8:B8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J71:J83" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J84:J98" type="list">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
v2 budget: final audit (links, sellers, tip wire price)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y1g5ouZCd4fvcL4KzTMSdf
</commit_message>
<xml_diff>
--- a/docs/v2-budget/STM_v2_budget.xlsx
+++ b/docs/v2-budget/STM_v2_budget.xlsx
@@ -548,7 +548,7 @@
     <t xml:space="preserve">New. Recommended by our design studies so scans are not limited to slow speeds.</t>
   </si>
   <si>
-    <t xml:space="preserve">100 megaohm resistor</t>
+    <t xml:space="preserve">Ohmite SM104031006FE</t>
   </si>
   <si>
     <t xml:space="preserve">5. Frame, sample holder and vibration isolation</t>
@@ -671,7 +671,7 @@
     <t xml:space="preserve">New. v1 used loose coins, which can shift and cause small jumps.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hardware store</t>
+    <t xml:space="preserve">Home Depot</t>
   </si>
   <si>
     <t xml:space="preserve">steel plate or bar offcuts</t>
@@ -1109,16 +1109,16 @@
     <t xml:space="preserve">Tip wire</t>
   </si>
   <si>
-    <t xml:space="preserve">Platinum-iridium wire, 0.25 mm thick. Each tip is cut from it with scissors; this metal stays sharp in air. Enough for dozens of tips.</t>
+    <t xml:space="preserve">Platinum-iridium wire, 0.25 mm thick, 20 cm long. Each tip is cut from it with scissors; this metal stays sharp in air. Enough for dozens of tips. Ships from the UK.</t>
   </si>
   <si>
     <t xml:space="preserve">Changed. v1 made its tips from tungsten wire, which corrodes in air. Replaces ready-made tips in the earlier budget at about the same price but many more tips.</t>
   </si>
   <si>
-    <t xml:space="preserve">Advent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt80/Ir20 wire, 0.25 mm, 0.2 m</t>
+    <t xml:space="preserve">Advent Research Materials</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT671004 (Pt80/Ir20, 0.25 mm, 0.2 m)</t>
   </si>
   <si>
     <t xml:space="preserve">Graphite test sample</t>
@@ -2627,11 +2627,11 @@
       <c r="B6" s="19"/>
       <c r="C6" s="20" t="n">
         <f aca="false">H159</f>
-        <v>2634.65</v>
+        <v>2668.88</v>
       </c>
       <c r="D6" s="21" t="n">
         <f aca="false">H160</f>
-        <v>1687.75</v>
+        <v>1694.7</v>
       </c>
       <c r="E6" s="21"/>
     </row>
@@ -2642,11 +2642,11 @@
       <c r="B7" s="19"/>
       <c r="C7" s="20" t="n">
         <f aca="false">H161</f>
-        <v>3307.765</v>
+        <v>3341.985</v>
       </c>
       <c r="D7" s="21" t="n">
         <f aca="false">H162</f>
-        <v>2360.855</v>
+        <v>2367.815</v>
       </c>
       <c r="E7" s="21"/>
     </row>
@@ -2657,7 +2657,7 @@
       <c r="B8" s="22"/>
       <c r="C8" s="23" t="n">
         <f aca="false">H154</f>
-        <v>2634.65</v>
+        <v>2668.88</v>
       </c>
       <c r="D8" s="24"/>
       <c r="E8" s="24"/>
@@ -3741,17 +3741,17 @@
         <v>2</v>
       </c>
       <c r="G53" s="30" t="n">
-        <v>3</v>
+        <v>5.73</v>
       </c>
       <c r="H53" s="30" t="n">
         <f aca="false">IF(K53="No",0,F53*G53)</f>
-        <v>6</v>
+        <v>11.46</v>
       </c>
       <c r="I53" s="33" t="s">
         <v>96</v>
       </c>
       <c r="J53" s="31" t="str">
-        <f aca="false">HYPERLINK("https://www.digikey.com/en/products/result?keywords=100M%20ohm%20resistor","Open")</f>
+        <f aca="false">HYPERLINK("https://octopart.com/search?q=SM104031006FE","Open")</f>
         <v>Open</v>
       </c>
       <c r="K53" s="32" t="s">
@@ -3770,7 +3770,7 @@
       <c r="G54" s="8"/>
       <c r="H54" s="9" t="n">
         <f aca="false">SUM(H48:H53)</f>
-        <v>92.37</v>
+        <v>97.83</v>
       </c>
       <c r="I54" s="8"/>
       <c r="J54" s="8"/>
@@ -4172,7 +4172,7 @@
         <v>220</v>
       </c>
       <c r="D67" s="29" t="s">
-        <v>216</v>
+        <v>88</v>
       </c>
       <c r="E67" s="28" t="s">
         <v>221</v>
@@ -4283,7 +4283,7 @@
         <v>233</v>
       </c>
       <c r="D70" s="29" t="s">
-        <v>216</v>
+        <v>88</v>
       </c>
       <c r="E70" s="28" t="s">
         <v>234</v>
@@ -4664,7 +4664,7 @@
       <c r="G86" s="35"/>
       <c r="H86" s="36" t="n">
         <f aca="false">H26+H37+H45+H54+H71+H77+H84</f>
-        <v>1171.19</v>
+        <v>1176.65</v>
       </c>
       <c r="I86" s="35"/>
       <c r="J86" s="35"/>
@@ -4727,7 +4727,7 @@
       <c r="E91" s="27"/>
       <c r="H91" s="30" t="n">
         <f aca="false">ROUND(0.08*(H42+H50+H51+H53+H81),2)</f>
-        <v>5.14</v>
+        <v>5.58</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4742,7 +4742,7 @@
       <c r="G92" s="35"/>
       <c r="H92" s="36" t="n">
         <f aca="false">SUM(H89:H91)</f>
-        <v>272.36</v>
+        <v>272.8</v>
       </c>
       <c r="I92" s="35"/>
       <c r="J92" s="35"/>
@@ -5773,17 +5773,17 @@
         <v>1</v>
       </c>
       <c r="G133" s="30" t="n">
-        <v>274</v>
+        <v>297</v>
       </c>
       <c r="H133" s="30" t="n">
         <f aca="false">IF(OR(K133="Yes",K133=TRUE()),0,F133*G133)</f>
-        <v>274</v>
-      </c>
-      <c r="I133" s="33" t="s">
-        <v>96</v>
+        <v>297</v>
+      </c>
+      <c r="I133" s="29" t="s">
+        <v>103</v>
       </c>
       <c r="J133" s="31" t="str">
-        <f aca="false">HYPERLINK("https://www.advent-rm.com/","Open")</f>
+        <f aca="false">HYPERLINK("https://www.advent-rm.com/en-GB/Products/Alloys/Platinum-Iridium/Form/Wire/Line/PT6710","Open")</f>
         <v>Open</v>
       </c>
       <c r="K133" s="53"/>
@@ -6255,7 +6255,7 @@
       <c r="G147" s="55"/>
       <c r="H147" s="56" t="n">
         <f aca="false">SUM(H133:H146)</f>
-        <v>798.91</v>
+        <v>821.91</v>
       </c>
       <c r="I147" s="55"/>
       <c r="J147" s="55"/>
@@ -6290,7 +6290,7 @@
       <c r="G150" s="59"/>
       <c r="H150" s="60" t="n">
         <f aca="false">H86+IF((K97="Yes"),H122,0)+H147</f>
-        <v>1970.1</v>
+        <v>1998.56</v>
       </c>
       <c r="I150" s="59"/>
       <c r="J150" s="59"/>
@@ -6308,7 +6308,7 @@
       <c r="G151" s="59"/>
       <c r="H151" s="60" t="n">
         <f aca="false">H92+IF((K97="Yes"),H128,0)</f>
-        <v>272.36</v>
+        <v>272.8</v>
       </c>
       <c r="I151" s="59"/>
       <c r="J151" s="59"/>
@@ -6328,7 +6328,7 @@
       <c r="G152" s="59"/>
       <c r="H152" s="60" t="n">
         <f aca="false">ROUND(H150*0.0775,2)</f>
-        <v>152.68</v>
+        <v>154.89</v>
       </c>
       <c r="I152" s="59"/>
       <c r="J152" s="59"/>
@@ -6348,7 +6348,7 @@
       <c r="G153" s="59"/>
       <c r="H153" s="60" t="n">
         <f aca="false">ROUND((H150+H151+H152)*0.1,2)</f>
-        <v>239.51</v>
+        <v>242.63</v>
       </c>
       <c r="I153" s="59"/>
       <c r="J153" s="59"/>
@@ -6366,7 +6366,7 @@
       <c r="G154" s="12"/>
       <c r="H154" s="13" t="n">
         <f aca="false">H150+H151+H152+H153</f>
-        <v>2634.65</v>
+        <v>2668.88</v>
       </c>
       <c r="I154" s="12"/>
       <c r="J154" s="12"/>
@@ -6386,7 +6386,7 @@
       <c r="G155" s="59"/>
       <c r="H155" s="60" t="n">
         <f aca="false">2000-H154</f>
-        <v>-634.65</v>
+        <v>-668.88</v>
       </c>
       <c r="I155" s="59"/>
       <c r="J155" s="59"/>
@@ -6429,24 +6429,24 @@
       <c r="B159" s="64"/>
       <c r="C159" s="6" t="n">
         <f aca="false">H86+SUMPRODUCT(F133:F146,G133:G146)</f>
-        <v>1970.1</v>
+        <v>1998.56</v>
       </c>
       <c r="D159" s="6" t="n">
         <f aca="false">H92</f>
-        <v>272.36</v>
+        <v>272.8</v>
       </c>
       <c r="E159" s="65" t="n">
         <f aca="false">ROUND(C159*0.0775,2)</f>
-        <v>152.68</v>
+        <v>154.89</v>
       </c>
       <c r="F159" s="65"/>
       <c r="G159" s="6" t="n">
         <f aca="false">ROUND((C159+D159+E159)*0.1,2)</f>
-        <v>239.51</v>
+        <v>242.63</v>
       </c>
       <c r="H159" s="66" t="n">
         <f aca="false">C159+D159+E159+G159</f>
-        <v>2634.65</v>
+        <v>2668.88</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6456,24 +6456,24 @@
       <c r="B160" s="64"/>
       <c r="C160" s="6" t="n">
         <f aca="false">H86</f>
-        <v>1171.19</v>
+        <v>1176.65</v>
       </c>
       <c r="D160" s="6" t="n">
         <f aca="false">H92</f>
-        <v>272.36</v>
+        <v>272.8</v>
       </c>
       <c r="E160" s="65" t="n">
         <f aca="false">ROUND(C160*0.0775,2)</f>
-        <v>90.77</v>
+        <v>91.19</v>
       </c>
       <c r="F160" s="65"/>
       <c r="G160" s="6" t="n">
         <f aca="false">ROUND((C160+D160+E160)*0.1,2)</f>
-        <v>153.43</v>
+        <v>154.06</v>
       </c>
       <c r="H160" s="66" t="n">
         <f aca="false">C160+D160+E160+G160</f>
-        <v>1687.75</v>
+        <v>1694.7</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6483,24 +6483,24 @@
       <c r="B161" s="64"/>
       <c r="C161" s="6" t="n">
         <f aca="false">H86+H122+SUMPRODUCT(F133:F146,G133:G146)</f>
-        <v>2382.215</v>
+        <v>2410.675</v>
       </c>
       <c r="D161" s="6" t="n">
         <f aca="false">H92+H128</f>
-        <v>440.22</v>
+        <v>440.66</v>
       </c>
       <c r="E161" s="65" t="n">
         <f aca="false">ROUND(C161*0.0775,2)</f>
-        <v>184.62</v>
+        <v>186.83</v>
       </c>
       <c r="F161" s="65"/>
       <c r="G161" s="6" t="n">
         <f aca="false">ROUND((C161+D161+E161)*0.1,2)</f>
-        <v>300.71</v>
+        <v>303.82</v>
       </c>
       <c r="H161" s="66" t="n">
         <f aca="false">C161+D161+E161+G161</f>
-        <v>3307.765</v>
+        <v>3341.985</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6510,24 +6510,24 @@
       <c r="B162" s="64"/>
       <c r="C162" s="6" t="n">
         <f aca="false">H86+H122</f>
-        <v>1583.305</v>
+        <v>1588.765</v>
       </c>
       <c r="D162" s="6" t="n">
         <f aca="false">H92+H128</f>
-        <v>440.22</v>
+        <v>440.66</v>
       </c>
       <c r="E162" s="65" t="n">
         <f aca="false">ROUND(C162*0.0775,2)</f>
-        <v>122.71</v>
+        <v>123.13</v>
       </c>
       <c r="F162" s="65"/>
       <c r="G162" s="6" t="n">
         <f aca="false">ROUND((C162+D162+E162)*0.1,2)</f>
-        <v>214.62</v>
+        <v>215.26</v>
       </c>
       <c r="H162" s="66" t="n">
         <f aca="false">C162+D162+E162+G162</f>
-        <v>2360.855</v>
+        <v>2367.815</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>